<commit_message>
Add Problem #130 and Consolidation & Surcharge Preload Lab with reclaimed lake/ditch context and 21-tab toolbox
</commit_message>
<xml_diff>
--- a/public/Civil_Engineering_Master_Toolbox.xlsx
+++ b/public/Civil_Engineering_Master_Toolbox.xlsx
@@ -27,6 +27,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50x50 Slab &amp; Helical Piles" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPSH &amp; Pump Cavitation" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stormwater &amp; TR-55 CN" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidation &amp; Surcharge" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -149,7 +150,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -185,55 +186,11 @@
         <color rgb="000F172A"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -430,8 +387,6 @@
     <xf numFmtId="164" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -797,13 +752,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="93" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="153" customWidth="1" min="4" max="4"/>
+    <col width="164" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -827,7 +782,7 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1. WORKBOOK NAVIGATION &amp; MODULE DIRECTORY (20 WORKSHEETS)</t>
+          <t>1. WORKBOOK NAVIGATION &amp; MODULE DIRECTORY (21 WORKSHEETS)</t>
         </is>
       </c>
     </row>
@@ -1271,205 +1226,205 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Consolidation &amp; Surcharge</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Geotechnical Soil Mechanics</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>NCEES § 3.3 &amp; § 3.4 • Terzaghi 1-D</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Time rate of consolidation, single vs double drainage (Hdr), Terzaghi Tv, preload surcharge design, required soil weight &amp; fill thickness to eliminate settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>2. STANDARDIZED COLOR CODING &amp; CELL CONVENTIONS</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>User Modifiable Input Parameter</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Soft Blue fill (#EFF6FF) with thin border. Modify these values to customize scenarios.</t>
         </is>
       </c>
-      <c r="C27" s="70" t="n"/>
-      <c r="D27" s="71" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Live Dynamic Excel Formula</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>White / Neutral cell containing real formulas (=SUM, =IF, =SQRT, etc.). Do not overwrite.</t>
         </is>
       </c>
-      <c r="C28" s="70" t="n"/>
-      <c r="D28" s="71" t="n"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Code Check / Design Status: PASS</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Soft Green fill (#DCFCE7) indicating compliance with NCEES, ACI, AASHTO, or OSHA criteria.</t>
         </is>
       </c>
-      <c r="C29" s="70" t="n"/>
-      <c r="D29" s="71" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>Code Check / Design Status: FAIL</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Soft Red fill (#FEE2E2) indicating safety factor violation or overtopping hazard.</t>
         </is>
       </c>
-      <c r="C30" s="70" t="n"/>
-      <c r="D30" s="71" t="n"/>
-    </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
+    </row>
+    <row r="32"/>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>3. NCEES CIVIL PE FREQUENT UNIT CONVERSIONS</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>1 acre-foot</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>43,560 ft³ = 325,851 gallons</t>
-        </is>
-      </c>
-      <c r="C33" s="70" t="n"/>
-      <c r="D33" s="71" t="n"/>
     </row>
     <row r="34" ht="19" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>1 ft³ of Water</t>
+          <t>1 acre-foot</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>7.48052 gallons = 62.4 lbs (at 60°F)</t>
-        </is>
-      </c>
-      <c r="C34" s="70" t="n"/>
-      <c r="D34" s="71" t="n"/>
+          <t>43,560 ft³ = 325,851 gallons</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="19" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>1 cubic foot per second (cfs)</t>
+          <t>1 ft³ of Water</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>448.83 gallons per minute (gpm) = 0.6463 MGD</t>
-        </is>
-      </c>
-      <c r="C35" s="70" t="n"/>
-      <c r="D35" s="71" t="n"/>
+          <t>7.48052 gallons = 62.4 lbs (at 60°F)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="19" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>1 psi pressure head</t>
+          <t>1 cubic foot per second (cfs)</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>2.307 feet of water column (ft H₂O)</t>
-        </is>
-      </c>
-      <c r="C36" s="70" t="n"/>
-      <c r="D36" s="71" t="n"/>
+          <t>448.83 gallons per minute (gpm) = 0.6463 MGD</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="19" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Standard Atmospheric Pressure (Sea Level)</t>
+          <t>1 psi pressure head</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>14.696 psia = 2,116 psf = 33.90 ft H₂O = 29.92 in Hg</t>
-        </is>
-      </c>
-      <c r="C37" s="70" t="n"/>
-      <c r="D37" s="71" t="n"/>
+          <t>2.307 feet of water column (ft H₂O)</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="19" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Acceleration of Gravity (g)</t>
+          <t>Standard Atmospheric Pressure (Sea Level)</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>32.174 ft/s² = 9.80665 m/s²</t>
-        </is>
-      </c>
-      <c r="C38" s="70" t="n"/>
-      <c r="D38" s="71" t="n"/>
+          <t>14.696 psia = 2,116 psf = 33.90 ft H₂O = 29.92 in Hg</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="19" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Density of Normal-Weight Concrete</t>
+          <t>Acceleration of Gravity (g)</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>145 to 150 lbs/ft³ (pcf)</t>
-        </is>
-      </c>
-      <c r="C39" s="70" t="n"/>
-      <c r="D39" s="71" t="n"/>
+          <t>32.174 ft/s² = 9.80665 m/s²</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="19" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
+          <t>Density of Normal-Weight Concrete</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>145 to 150 lbs/ft³ (pcf)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="19" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
           <t>Modulus of Elasticity of Steel (Es)</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>29,000,000 psi (29,000 ksi)</t>
         </is>
       </c>
-      <c r="C40" s="70" t="n"/>
-      <c r="D40" s="71" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A32:G32"/>
     <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B33:D33"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B37:D37"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B41:D41"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="B40:D40"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B39:D39"/>
+    <mergeCell ref="A33:G33"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="B34:D34"/>
   </mergeCells>
@@ -1680,6 +1635,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -1716,7 +1672,7 @@
         </is>
       </c>
       <c r="B16" s="30">
-        <f>((B6 * B6^3) / (12 * (1 - B7^2) * B8))^(0.25)</f>
+        <f>((B6 * B4^3) / (12 * (1 - B7^2) * B8))^(0.25)</f>
         <v/>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -1737,7 +1693,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>IF(B10 &lt; 1.724*B6, SQRT(1.6*B10^2 + B6^2) - 0.675*B6, B10)</f>
+        <f>IF(B10 &lt; 1.724*B4, SQRT(1.6*B10^2 + B4^2) - 0.675*B4, B10)</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -1772,6 +1728,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -1813,7 +1770,7 @@
         </is>
       </c>
       <c r="B22" s="39">
-        <f>(3 * B9 * (1 + B7) / (2 * PI() * B6^2)) * (LN(B12 / B13) + 0.6159)</f>
+        <f>(3 * B9 * (1 + B7) / (2 * PI() * B4^2)) * (LN(B12 / B13) + 0.6159)</f>
         <v/>
       </c>
       <c r="C22" s="57">
@@ -1836,7 +1793,7 @@
         </is>
       </c>
       <c r="B23" s="39">
-        <f>(0.529 * B9 * (1 + 0.54*B7) / B6^2) * (LOG10(B6 * B6^3 / (B8 * B13^4)) - 0.71)</f>
+        <f>(0.529 * B9 * (1 + 0.54*B7) / B4^2) * (LOG10(B6 * B4^3 / (B8 * B13^4)) - 0.71)</f>
         <v/>
       </c>
       <c r="C23" s="57">
@@ -1859,7 +1816,7 @@
         </is>
       </c>
       <c r="B24" s="39">
-        <f>(3 * B9 / B6^2) * (1 - (B10 * SQRT(2) / B12)^0.6)</f>
+        <f>(3 * B9 / B4^2) * (1 - (B10 * SQRT(2) / B12)^0.6)</f>
         <v/>
       </c>
       <c r="C24" s="57">
@@ -2016,7 +1973,7 @@
         </is>
       </c>
       <c r="B9" s="30">
-        <f>B6 - B8</f>
+        <f>B4 - B6</f>
         <v/>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -2585,6 +2542,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -2621,7 +2579,7 @@
         </is>
       </c>
       <c r="B16" s="60">
-        <f>(B7 * 12 * B7^3) / 12</f>
+        <f>(B5 * 12 * B7^3) / 12</f>
         <v/>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -2642,7 +2600,7 @@
         </is>
       </c>
       <c r="B17" s="60">
-        <f>(4 * B10 * B12) / (B6 * 12)</f>
+        <f>(4 * B10 * B12) / (B4 * 12)</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -2726,7 +2684,7 @@
         </is>
       </c>
       <c r="B21" s="60">
-        <f>2 * (9 * B10 * B16) / ((B7 * 12) * (1 - B9/(B7*12))^3)</f>
+        <f>2 * (9 * B10 * B16) / ((B5 * 12) * (1 - B9/(B5*12))^3)</f>
         <v/>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -2740,6 +2698,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -2839,7 +2798,7 @@
         </is>
       </c>
       <c r="B28" s="60">
-        <f>(120.0 * B7 * B6^2) / 12</f>
+        <f>(120.0 * B5 * B4^2) / 12</f>
         <v/>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -3088,6 +3047,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -3154,11 +3114,11 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>(B7/2) * (SQRT(3*(B6/B7)^2*C12 + 1) - 1)</f>
+        <f>(B5/2) * (SQRT(3*(B4/B5)^2*C12 + 1) - 1)</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>(B7/2) * (SQRT(3*(B6/B7)^2*C12 + 1) - 1)</f>
+        <f>(B5/2) * (SQRT(3*(B4/B5)^2*C12 + 1) - 1)</f>
         <v/>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -3184,7 +3144,7 @@
         </is>
       </c>
       <c r="C18" s="20">
-        <f>2 * (B6*(1+B8)*B7/D13 + B7*(1+B9)*B6/(B7/2))</f>
+        <f>2 * (B6*(1+B8)*B5/D13 + B7*(1+B9)*B4/(B5/2))</f>
         <v/>
       </c>
       <c r="D18" s="18" t="inlineStr">
@@ -3210,7 +3170,7 @@
         </is>
       </c>
       <c r="C19" s="20">
-        <f>(B6*B7/6) * (3 - 2*D13/B6)</f>
+        <f>(B4*B5/6) * (3 - 2*D13/B4)</f>
         <v/>
       </c>
       <c r="D19" s="18" t="inlineStr">
@@ -3249,6 +3209,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -3523,6 +3484,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -3564,18 +3526,18 @@
         </is>
       </c>
       <c r="B16" s="30">
-        <f>(B9 * B6^2) / 8</f>
+        <f>(B9 * B4^2) / 8</f>
         <v/>
       </c>
       <c r="C16" s="20">
-        <f>(B9 * B6^2) / 8</f>
+        <f>(B9 * B4^2) / 8</f>
         <v/>
       </c>
       <c r="D16" s="30" t="n">
         <v>6.5</v>
       </c>
       <c r="E16" s="30">
-        <f>((B9 * B6^2) / 8) * 12 / (0.90 * 60000 * 0.90 * D13)</f>
+        <f>((B9 * B4^2) / 8) * 12 / (0.90 * 60000 * 0.90 * D13)</f>
         <v/>
       </c>
     </row>
@@ -3645,6 +3607,7 @@
         <v/>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -4000,7 +3963,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>MAX(B7, B8) / MIN(B7, B8)</f>
+        <f>MAX(B5, B6) / MIN(B5, B6)</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -4021,7 +3984,7 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>2*(B7 + B6) + 2*(B8 + B6)</f>
+        <f>2*(B5 + B4) + 2*(B6 + B4)</f>
         <v/>
       </c>
       <c r="C18" s="54" t="inlineStr">
@@ -4042,7 +4005,7 @@
         </is>
       </c>
       <c r="B19" s="22">
-        <f>B18 * B6</f>
+        <f>B15 * B4</f>
         <v/>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -4098,7 +4061,7 @@
         </is>
       </c>
       <c r="C23" s="20">
-        <f>(2 + 4/B17) * B12 * SQRT(B11) * B18 * B6 / 1000</f>
+        <f>(2 + 4/B14) * B10 * SQRT(B9) * B15 * B4 / 1000</f>
         <v/>
       </c>
       <c r="D23" s="14" t="inlineStr">
@@ -4119,7 +4082,7 @@
         </is>
       </c>
       <c r="C24" s="20">
-        <f>(B10 * B6 / B18 + 2) * B12 * SQRT(B11) * B18 * B6 / 1000</f>
+        <f>(B8 * B4 / B15 + 2) * B10 * SQRT(B9) * B15 * B4 / 1000</f>
         <v/>
       </c>
       <c r="D24" s="14" t="inlineStr">
@@ -4140,7 +4103,7 @@
         </is>
       </c>
       <c r="C25" s="20">
-        <f>4 * B12 * SQRT(B11) * B18 * B6 / 1000</f>
+        <f>4 * B10 * SQRT(B9) * B15 * B4 / 1000</f>
         <v/>
       </c>
       <c r="D25" s="14" t="inlineStr">
@@ -4161,7 +4124,7 @@
         </is>
       </c>
       <c r="C26" s="25">
-        <f>MIN(C23, C24, C25)</f>
+        <f>MIN(C19, C20, C21)</f>
         <v/>
       </c>
       <c r="D26" s="44" t="inlineStr">
@@ -4182,7 +4145,7 @@
         </is>
       </c>
       <c r="C27" s="25">
-        <f>0.75 * C26</f>
+        <f>0.75 * C22</f>
         <v/>
       </c>
       <c r="D27" s="44" t="inlineStr">
@@ -4256,11 +4219,11 @@
         </is>
       </c>
       <c r="B32" s="39">
-        <f>(B13 * 1000) / (B18 * B6)</f>
+        <f>(B11 * 1000) / (B15 * B4)</f>
         <v/>
       </c>
       <c r="C32" s="57">
-        <f>0.75 * (C26 * 1000) / (B18 * B6)</f>
+        <f>0.75 * (C22 * 1000) / (B15 * B4)</f>
         <v/>
       </c>
       <c r="D32" s="41">
@@ -4488,6 +4451,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -4572,6 +4536,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -4969,6 +4934,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -5138,6 +5104,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -5284,6 +5251,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
@@ -5538,7 +5506,7 @@
         </is>
       </c>
       <c r="B8" s="22">
-        <f>B6 * B7</f>
+        <f>B4 * B5</f>
         <v/>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -6196,6 +6164,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -6471,6 +6440,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
@@ -6900,6 +6870,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -6941,11 +6912,11 @@
         </is>
       </c>
       <c r="B20" s="19">
-        <f>(1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7)))</f>
+        <f>(1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5)))</f>
         <v/>
       </c>
       <c r="C20" s="20">
-        <f>ROUND((1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7))), 4)</f>
+        <f>ROUND((1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5))), 4)</f>
         <v/>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -6966,19 +6937,19 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>0.5 * B8 * B6^2 * B20</f>
+        <f>0.5 * B6 * B4^2 * C18</f>
         <v/>
       </c>
       <c r="C21" s="20">
-        <f>0.5 * B8 * B6^2 * ((1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7))))</f>
+        <f>0.5 * B6 * B4^2 * ((1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5))))</f>
         <v/>
       </c>
       <c r="D21" s="22">
-        <f>B6 / 3</f>
+        <f>B4 / 3</f>
         <v/>
       </c>
       <c r="E21" s="22">
-        <f>C21 * D21</f>
+        <f>C19 * D19</f>
         <v/>
       </c>
     </row>
@@ -6989,19 +6960,19 @@
         </is>
       </c>
       <c r="B22" s="22">
-        <f>B13 * B6 * B20</f>
+        <f>B11 * B4 * C18</f>
         <v/>
       </c>
       <c r="C22" s="20">
-        <f>B13 * B6 * ((1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7))))</f>
+        <f>B11 * B4 * ((1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5))))</f>
         <v/>
       </c>
       <c r="D22" s="22">
-        <f>B6 / 2</f>
+        <f>B4 / 2</f>
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>C22 * D22</f>
+        <f>C20 * D20</f>
         <v/>
       </c>
     </row>
@@ -7017,7 +6988,7 @@
         </is>
       </c>
       <c r="C23" s="25">
-        <f>C21 + C22</f>
+        <f>C19 + C20</f>
         <v/>
       </c>
       <c r="D23" s="24" t="inlineStr">
@@ -7026,10 +6997,11 @@
         </is>
       </c>
       <c r="E23" s="26">
-        <f>E21 + E22</f>
-        <v/>
-      </c>
-    </row>
+        <f>E19 + E20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
@@ -7071,19 +7043,19 @@
         </is>
       </c>
       <c r="B27" s="22">
-        <f>(B6 - B10) * B11 * B14</f>
+        <f>(B4 - B8) * B9 * B12</f>
         <v/>
       </c>
       <c r="C27" s="20">
-        <f>(B6 - B10) * B11 * B14</f>
+        <f>(B4 - B8) * B9 * B12</f>
         <v/>
       </c>
       <c r="D27" s="22">
-        <f>B12 + B11/2</f>
+        <f>B10 + B9/2</f>
         <v/>
       </c>
       <c r="E27" s="22">
-        <f>C27 * D27</f>
+        <f>C24 * D24</f>
         <v/>
       </c>
     </row>
@@ -7094,19 +7066,19 @@
         </is>
       </c>
       <c r="B28" s="22">
-        <f>B9 * B10 * B14</f>
+        <f>B7 * B8 * B12</f>
         <v/>
       </c>
       <c r="C28" s="20">
-        <f>B9 * B10 * B14</f>
+        <f>B7 * B8 * B12</f>
         <v/>
       </c>
       <c r="D28" s="22">
-        <f>B9 / 2</f>
+        <f>B7 / 2</f>
         <v/>
       </c>
       <c r="E28" s="22">
-        <f>C28 * D28</f>
+        <f>C25 * D25</f>
         <v/>
       </c>
     </row>
@@ -7117,19 +7089,19 @@
         </is>
       </c>
       <c r="B29" s="22">
-        <f>(B9 - B12 - B11) * (B6 - B10) * B8</f>
+        <f>(B7 - B10 - B9) * (B4 - B8) * B6</f>
         <v/>
       </c>
       <c r="C29" s="20">
-        <f>(B9 - B12 - B11) * (B6 - B10) * B8</f>
+        <f>(B7 - B10 - B9) * (B4 - B8) * B6</f>
         <v/>
       </c>
       <c r="D29" s="22">
-        <f>B9 - (B9 - B12 - B11)/2</f>
+        <f>B7 - (B7 - B10 - B9)/2</f>
         <v/>
       </c>
       <c r="E29" s="22">
-        <f>C29 * D29</f>
+        <f>C26 * D26</f>
         <v/>
       </c>
     </row>
@@ -7145,7 +7117,7 @@
         </is>
       </c>
       <c r="C30" s="25">
-        <f>C27 + C28 + C29</f>
+        <f>C24 + C25 + C26</f>
         <v/>
       </c>
       <c r="D30" s="24" t="inlineStr">
@@ -7154,10 +7126,11 @@
         </is>
       </c>
       <c r="E30" s="26">
-        <f>E27 + E28 + E29</f>
-        <v/>
-      </c>
-    </row>
+        <f>E24 + E25 + E26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
@@ -7199,7 +7172,7 @@
         </is>
       </c>
       <c r="B34" s="27">
-        <f>E30 / E23</f>
+        <f>E27 / E21</f>
         <v/>
       </c>
       <c r="C34" s="28" t="inlineStr">
@@ -7208,11 +7181,11 @@
         </is>
       </c>
       <c r="D34" s="29">
-        <f>E30 / E23</f>
+        <f>E27 / E21</f>
         <v/>
       </c>
       <c r="E34" s="29">
-        <f>IF(B34&gt;=2.0, "PASS - OVERTURNING SAFE", "FAIL - UNDERSIZED TOE")</f>
+        <f>IF(B30&gt;=2.0, "PASS - OVERTURNING SAFE", "FAIL - UNDERSIZED TOE")</f>
         <v/>
       </c>
     </row>
@@ -7223,7 +7196,7 @@
         </is>
       </c>
       <c r="B35" s="27">
-        <f>(C30 * B15) / C23</f>
+        <f>(C27 * B13) / C21</f>
         <v/>
       </c>
       <c r="C35" s="28" t="inlineStr">
@@ -7232,11 +7205,11 @@
         </is>
       </c>
       <c r="D35" s="29">
-        <f>(C30 * B15) / C23</f>
+        <f>(C27 * B13) / C21</f>
         <v/>
       </c>
       <c r="E35" s="29">
-        <f>IF(B35&gt;=1.5, "PASS - SLIDING SAFE", "FAIL - ADD SHEAR KEY")</f>
+        <f>IF(B31&gt;=1.5, "PASS - SLIDING SAFE", "FAIL - ADD SHEAR KEY")</f>
         <v/>
       </c>
     </row>
@@ -7247,7 +7220,7 @@
         </is>
       </c>
       <c r="B36" s="30">
-        <f>(E30 - E23) / C30</f>
+        <f>(E27 - E21) / C27</f>
         <v/>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -7255,9 +7228,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D36" s="14">
-        <f>(E30 - E23) / C30</f>
-        <v/>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>x_bar = (M_r - M_ot) / W</t>
+        </is>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
@@ -7272,7 +7246,7 @@
         </is>
       </c>
       <c r="B37" s="27">
-        <f>ABS(B9/2 - B36)</f>
+        <f>ABS(B7/2 - B32)</f>
         <v/>
       </c>
       <c r="C37" s="28" t="inlineStr">
@@ -7281,11 +7255,11 @@
         </is>
       </c>
       <c r="D37" s="29">
-        <f>B9/6</f>
+        <f>B7/6</f>
         <v/>
       </c>
       <c r="E37" s="29">
-        <f>IF(B37&lt;=(B9/6), "PASS - WITHIN MIDDLE THIRD (KERN)", "FAIL - TENSION AT HEEL")</f>
+        <f>IF(B33&lt;=(B7/6), "PASS - WITHIN MIDDLE THIRD (KERN)", "FAIL - TENSION AT HEEL")</f>
         <v/>
       </c>
     </row>
@@ -7296,7 +7270,7 @@
         </is>
       </c>
       <c r="B38" s="31">
-        <f>(C30 / B9) * (1 + 6*B37/B9)</f>
+        <f>(C27 / B7) * (1 + 6*B33/B7)</f>
         <v/>
       </c>
       <c r="C38" s="28" t="inlineStr">
@@ -7305,11 +7279,11 @@
         </is>
       </c>
       <c r="D38" s="32">
-        <f>B16 - B38</f>
+        <f>B14 - B34</f>
         <v/>
       </c>
       <c r="E38" s="32">
-        <f>IF(B38&lt;=B16, "PASS - BEARING CAPACITY ADEQUATE", "FAIL - EXCEEDS BEARING CAPACITY")</f>
+        <f>IF(B34&lt;=B14, "PASS - BEARING CAPACITY ADEQUATE", "FAIL - EXCEEDS BEARING CAPACITY")</f>
         <v/>
       </c>
     </row>
@@ -7495,9 +7469,10 @@
           <t>COMPOSITE CURVE NUMBER (CN)</t>
         </is>
       </c>
-      <c r="B10" s="68">
-        <f>(B6*0.25 + B7*0.35 + B8*0.25 + B9*0.15)</f>
-        <v/>
+      <c r="B10" s="68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
@@ -7505,7 +7480,7 @@
         </is>
       </c>
       <c r="D10" s="69">
-        <f>SUM(D6:D7)</f>
+        <f>SUM(D4:D7)</f>
         <v/>
       </c>
       <c r="E10" s="68" t="inlineStr">
@@ -7514,6 +7489,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -7709,6 +7685,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -7862,6 +7839,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
@@ -8035,6 +8013,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42" ht="24" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
@@ -8281,6 +8260,1050 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A42:G42"/>
     <mergeCell ref="A23:G23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="74" customWidth="1" min="1" max="1"/>
+    <col width="71" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="63" customWidth="1" min="4" max="4"/>
+    <col width="107" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SOLVEDIN6 CIVIL MASTER TOOLBOX - TAB 21: TIME RATE OF CONSOLIDATION &amp; SOIL SURCHARGE PRELOAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NCEES PE Civil § 3.3 &amp; § 3.4 • Reclaimed Lake Bed / Filled Ditch Surcharge Preload &amp; Moisture Dissipation Solver</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1. IN-SITU COMPRESSIBLE SOIL STRATIGRAPHY &amp; GEOTECHNICAL PROPERTIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Stratigraphy &amp; Soil Parameter</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Design Value</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>NCEES Handbook Formulation / Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Compressible Clay Layer Total Thickness (H)</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Total saturated clay layer thickness</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Drainage Boundary Condition</t>
+        </is>
+      </c>
+      <c r="B7" s="65" t="inlineStr">
+        <is>
+          <t>Double Drainage</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Double (sand top/bottom) or Single (rock at bottom)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Maximum Drainage Path Distance (H_dr)</t>
+        </is>
+      </c>
+      <c r="B8" s="30">
+        <f>IF(B7="Single Drainage", B6, B6/2)</f>
+        <v/>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>H_dr = H/2 for double drainage, H for single drainage</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Coefficient of Consolidation (c_v)</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>ft²/day</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>Hydraulic consolidation rate property</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Clay Compression Index (C_c)</t>
+        </is>
+      </c>
+      <c r="B10" s="50" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>Slope of e vs log(sigma) virgin compression curve</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Initial In-Situ Void Ratio (e_0)</t>
+        </is>
+      </c>
+      <c r="B11" s="50" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>Initial volumetric void ratio of clay stratum</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Initial Effective Overburden Stress (σ'_v0)</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>2200</v>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>psf</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Effective vertical stress at mid-depth of clay layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2. STRUCTURAL FOUNDATION LOADING &amp; ULTIMATE SETTLEMENT (S_p,ult)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Structural Loading Parameter</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Design Value</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Governing Compression Equation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Foundation Footprint Length (L)</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Building / foundation footprint length</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Foundation Footprint Width (W)</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Building / foundation footprint width</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Total Foundation Footprint Area (A)</t>
+        </is>
+      </c>
+      <c r="B18" s="22">
+        <f>B16 * B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>sq ft</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>A = L * W</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Permanent Foundation Bearing Pressure (Δσ_p)</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>psf</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Net structural stress increase applied to soil</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Total Mid-Depth Vertical Stress (σ'_v0 + Δσ_p)</t>
+        </is>
+      </c>
+      <c r="B20" s="22">
+        <f>B12 + B19</f>
+        <v/>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>psf</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Total effective stress under permanent building load</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Clay Compression Factor [C_c * H / (1 + e_0)]</t>
+        </is>
+      </c>
+      <c r="B21" s="19">
+        <f>(B10 * B6) / (1 + B11)</f>
+        <v/>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>Dimensional coefficient for 1D settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Ultimate Primary Consolidation Settlement (S_p,ult)</t>
+        </is>
+      </c>
+      <c r="B22" s="19">
+        <f>B21 * LOG10(B20 / B12)</f>
+        <v/>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>S_p,ult = [Cc*H/(1+e0)] * log10((σ'v0 + Δσp) / σ'v0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>ULTIMATE PRIMARY SETTLEMENT IN INCHES</t>
+        </is>
+      </c>
+      <c r="B23" s="45">
+        <f>B22 * 12</f>
+        <v/>
+      </c>
+      <c r="C23" s="54" t="inlineStr">
+        <is>
+          <t>inches</t>
+        </is>
+      </c>
+      <c r="D23" s="44" t="inlineStr">
+        <is>
+          <t>Total moisture expulsion deformation to eliminate</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>3. PRELOAD SURCHARGE DESIGN: TIME ➔ REQUIRED SOIL WEIGHT (MODE A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Preload Surcharge Parameter</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Design Value</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Terzaghi 1-D Consolidation Derivation</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Allotted Preloading Time Window (t)</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n">
+        <v>180</v>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Target construction window before building erection</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Equivalent Preload Duration in Months</t>
+        </is>
+      </c>
+      <c r="B28" s="56">
+        <f>B27 / 30.4375</f>
+        <v/>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Duration in calendar months</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Terzaghi Time Factor (T_v)</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>(B9 * B27) / (B8^2)</f>
+        <v/>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="inlineStr">
+        <is>
+          <t>T_v = (c_v * t) / (H_dr^2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Degree of Consolidation under Preload (U_s)</t>
+        </is>
+      </c>
+      <c r="B30" s="19">
+        <f>IF(B29&lt;=0.2827, SQRT((4*B29)/PI()), 1 - 10^((1.781-B29)/0.933 - 2))</f>
+        <v/>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Terzaghi average consolidation ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Pore Water Moisture Dissipated Percentage</t>
+        </is>
+      </c>
+      <c r="B31" s="56">
+        <f>B30 * 100</f>
+        <v/>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Moisture squeezed out of clay pores in allotted time</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Required Ultimate Settlement under Preload</t>
+        </is>
+      </c>
+      <c r="B32" s="19">
+        <f>B22 / B30</f>
+        <v/>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>S_total,ult = S_p,ult / U_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Required Surcharge Soil Pressure (Δσ_s)</t>
+        </is>
+      </c>
+      <c r="B33" s="22">
+        <f>B12 * (10^(B32 / B21)) - B12 - B19</f>
+        <v/>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>psf</t>
+        </is>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>Additional vertical stress required to accelerate settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Surcharge Soil Compacted Unit Weight (γ_fill)</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n">
+        <v>125</v>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>pcf</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Compacted density of borrow soil surcharge</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>REQUIRED SURCHARGE FILL HEIGHT (h_s)</t>
+        </is>
+      </c>
+      <c r="B35" s="45">
+        <f>B33 / B34</f>
+        <v/>
+      </c>
+      <c r="C35" s="54" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D35" s="44" t="inlineStr">
+        <is>
+          <t>h_s = Δσ_s / γ_fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>Total Surcharge Fill Volume in Cubic Feet</t>
+        </is>
+      </c>
+      <c r="B36" s="22">
+        <f>B18 * B35</f>
+        <v/>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>cu ft</t>
+        </is>
+      </c>
+      <c r="D36" s="18" t="inlineStr">
+        <is>
+          <t>Volume = Area * h_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Total Surcharge Fill Volume in Cubic Yards</t>
+        </is>
+      </c>
+      <c r="B37" s="22">
+        <f>B36 / 27</f>
+        <v/>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>cu yd</t>
+        </is>
+      </c>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>Volume in bank / compacted cubic yards</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL SURCHARGE SOIL WEIGHT IN POUNDS</t>
+        </is>
+      </c>
+      <c r="B38" s="22">
+        <f>B36 * B34</f>
+        <v/>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>lbs</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>Weight = Volume * γ_fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>TOTAL SURCHARGE SOIL WEIGHT IN TONS</t>
+        </is>
+      </c>
+      <c r="B39" s="26">
+        <f>B38 / 2000</f>
+        <v/>
+      </c>
+      <c r="C39" s="54" t="inlineStr">
+        <is>
+          <t>Tons</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Required surcharge borrow weight in short tons</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>4. REVERSE SOLVER: SPECIFIED SURCHARGE WEIGHT ➔ PRELOAD TIME (MODE B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Reverse Solver Parameter</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Design Value</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Inverted Terzaghi Formulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>Specified Surcharge Soil Fill Height</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>Pre-selected contractor fill thickness</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>Generated Surcharge Effective Stress</t>
+        </is>
+      </c>
+      <c r="B44" s="22">
+        <f>B43 * B34</f>
+        <v/>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>psf</t>
+        </is>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>Δσ_s = h_s * γ_fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Total Surcharge Weight Placed in Tons</t>
+        </is>
+      </c>
+      <c r="B45" s="22">
+        <f>(B18 * B43 * B34) / 2000</f>
+        <v/>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>Tons</t>
+        </is>
+      </c>
+      <c r="D45" s="18" t="inlineStr">
+        <is>
+          <t>Total weight of 8.0-ft fill over footprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>Total Vertical Stress under 8-ft Surcharge</t>
+        </is>
+      </c>
+      <c r="B46" s="22">
+        <f>B12 + B19 + B44</f>
+        <v/>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>psf</t>
+        </is>
+      </c>
+      <c r="D46" s="18" t="inlineStr">
+        <is>
+          <t>σ'_v0 + Δσ_p + Δσ_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>Total Ultimate Settlement under 8-ft Fill</t>
+        </is>
+      </c>
+      <c r="B47" s="19">
+        <f>B21 * LOG10(B46 / B12)</f>
+        <v/>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>ft</t>
+        </is>
+      </c>
+      <c r="D47" s="21" t="inlineStr">
+        <is>
+          <t>Total settlement if load left permanently</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Required Consolidation Ratio (U_s,req)</t>
+        </is>
+      </c>
+      <c r="B48" s="19">
+        <f>B22 / B47</f>
+        <v/>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="21" t="inlineStr">
+        <is>
+          <t>U_s = S_p,ult / S_total,ult</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Required Terzaghi Time Factor (T_v,b)</t>
+        </is>
+      </c>
+      <c r="B49" s="19">
+        <f>1.781 - 0.933 * LOG10(100 - 100 * B48)</f>
+        <v/>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="21" t="inlineStr">
+        <is>
+          <t>T_v for U &gt; 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="23" t="inlineStr">
+        <is>
+          <t>REQUIRED PRELOADING DURATION IN DAYS</t>
+        </is>
+      </c>
+      <c r="B50" s="69">
+        <f>(B49 * (B8^2)) / B9</f>
+        <v/>
+      </c>
+      <c r="C50" s="54" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="D50" s="68" t="inlineStr">
+        <is>
+          <t>t = (T_v * H_dr^2) / c_v</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="23" t="inlineStr">
+        <is>
+          <t>REQUIRED PRELOADING DURATION IN MONTHS</t>
+        </is>
+      </c>
+      <c r="B51" s="69">
+        <f>B50 / 30.4375</f>
+        <v/>
+      </c>
+      <c r="C51" s="54" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D51" s="68" t="inlineStr">
+        <is>
+          <t>Duration in calendar months</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>5. FOUNDATION PERFORMANCE, PRECONSOLIDATION &amp; RESIDUAL SETTLEMENT CHECK</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Performance Check Parameter</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Design Value</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Criterion / Code Limit</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Status Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>Post-Construction Residual Settlement</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>inches</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Target = 0.00 inches (Fully dissipated)</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>PASS - SETTLEMENT ELIMINATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>Preconsolidation Stress Created (σ'_p)</t>
+        </is>
+      </c>
+      <c r="B56" s="22">
+        <f>B12 + B19 + B33</f>
+        <v/>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>psf</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Maximum past effective stress induced by preload</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>Overconsolidation Ratio (OCR)</t>
+        </is>
+      </c>
+      <c r="B57" s="27">
+        <f>(B12 + B19 + B33) / (B12 + B19)</f>
+        <v/>
+      </c>
+      <c r="C57" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="36" t="inlineStr">
+        <is>
+          <t>OCR = (σ'v0 + Δσp + Δσs) / (σ'v0 + Δσp)</t>
+        </is>
+      </c>
+      <c r="E57" s="29">
+        <f>IF(((B12+B19+B33)/(B12+B19))&gt;1.0, "PASS - OVERCONSOLIDATED STATE ACHIEVED", "FAIL - UNDERCONSOLIDATED")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A41:G41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8415,7 +9438,7 @@
         </is>
       </c>
       <c r="B9" s="33">
-        <f>B6 * B7 * B8</f>
+        <f>B4 * B5 * B6</f>
         <v/>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -8456,7 +9479,7 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>B9 * (B10 * 60)</f>
+        <f>B7 * (B8 * 60)</f>
         <v/>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -8477,7 +9500,7 @@
         </is>
       </c>
       <c r="B12" s="30">
-        <f>B11 / 43560</f>
+        <f>B9 / 43560</f>
         <v/>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -8491,6 +9514,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -8564,27 +9588,27 @@
         <v>1</v>
       </c>
       <c r="B17" s="22">
-        <f>120 + 2*3*A17</f>
+        <f>120 + 2*3*A14</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>60 + 2*3*A17</f>
+        <f>60 + 2*3*A14</f>
         <v/>
       </c>
       <c r="D17" s="22">
-        <f>B17 * C17</f>
+        <f>B14 * C14</f>
         <v/>
       </c>
       <c r="E17" s="22">
-        <f>(1/3)*(D16 + D17 + SQRT(D16*D17))</f>
+        <f>(1/3)*(D13 + D14 + SQRT(D13*D14))</f>
         <v/>
       </c>
       <c r="F17" s="20">
-        <f>E17</f>
+        <f>E14</f>
         <v/>
       </c>
       <c r="G17" s="20">
-        <f>F17/43560</f>
+        <f>F14/43560</f>
         <v/>
       </c>
     </row>
@@ -8593,27 +9617,27 @@
         <v>2</v>
       </c>
       <c r="B18" s="22">
-        <f>120 + 2*3*A18</f>
+        <f>120 + 2*3*A15</f>
         <v/>
       </c>
       <c r="C18" s="20">
-        <f>60 + 2*3*A18</f>
+        <f>60 + 2*3*A15</f>
         <v/>
       </c>
       <c r="D18" s="22">
-        <f>B18 * C18</f>
+        <f>B15 * C15</f>
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>(1/3)*(D17 + D18 + SQRT(D17*D18))</f>
+        <f>(1/3)*(D14 + D15 + SQRT(D14*D15))</f>
         <v/>
       </c>
       <c r="F18" s="20">
-        <f>F17 + E18</f>
+        <f>F14 + E15</f>
         <v/>
       </c>
       <c r="G18" s="20">
-        <f>F18/43560</f>
+        <f>F15/43560</f>
         <v/>
       </c>
     </row>
@@ -8622,27 +9646,27 @@
         <v>3</v>
       </c>
       <c r="B19" s="22">
-        <f>120 + 2*3*A19</f>
+        <f>120 + 2*3*A16</f>
         <v/>
       </c>
       <c r="C19" s="20">
-        <f>60 + 2*3*A19</f>
+        <f>60 + 2*3*A16</f>
         <v/>
       </c>
       <c r="D19" s="22">
-        <f>B19 * C19</f>
+        <f>B16 * C16</f>
         <v/>
       </c>
       <c r="E19" s="22">
-        <f>(1/3)*(D18 + D19 + SQRT(D18*D19))</f>
+        <f>(1/3)*(D15 + D16 + SQRT(D15*D16))</f>
         <v/>
       </c>
       <c r="F19" s="20">
-        <f>F18 + E19</f>
+        <f>F15 + E16</f>
         <v/>
       </c>
       <c r="G19" s="20">
-        <f>F19/43560</f>
+        <f>F16/43560</f>
         <v/>
       </c>
     </row>
@@ -8651,27 +9675,27 @@
         <v>4</v>
       </c>
       <c r="B20" s="22">
-        <f>120 + 2*3*A20</f>
+        <f>120 + 2*3*A17</f>
         <v/>
       </c>
       <c r="C20" s="20">
-        <f>60 + 2*3*A20</f>
+        <f>60 + 2*3*A17</f>
         <v/>
       </c>
       <c r="D20" s="22">
-        <f>B20 * C20</f>
+        <f>B17 * C17</f>
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>(1/3)*(D19 + D20 + SQRT(D19*D20))</f>
+        <f>(1/3)*(D16 + D17 + SQRT(D16*D17))</f>
         <v/>
       </c>
       <c r="F20" s="20">
-        <f>F19 + E20</f>
+        <f>F16 + E17</f>
         <v/>
       </c>
       <c r="G20" s="20">
-        <f>F20/43560</f>
+        <f>F17/43560</f>
         <v/>
       </c>
     </row>
@@ -8680,27 +9704,27 @@
         <v>5</v>
       </c>
       <c r="B21" s="22">
-        <f>120 + 2*3*A21</f>
+        <f>120 + 2*3*A18</f>
         <v/>
       </c>
       <c r="C21" s="20">
-        <f>60 + 2*3*A21</f>
+        <f>60 + 2*3*A18</f>
         <v/>
       </c>
       <c r="D21" s="22">
-        <f>B21 * C21</f>
+        <f>B18 * C18</f>
         <v/>
       </c>
       <c r="E21" s="22">
-        <f>(1/3)*(D20 + D21 + SQRT(D20*D21))</f>
+        <f>(1/3)*(D17 + D18 + SQRT(D17*D18))</f>
         <v/>
       </c>
       <c r="F21" s="20">
-        <f>F20 + E21</f>
+        <f>F17 + E18</f>
         <v/>
       </c>
       <c r="G21" s="20">
-        <f>F21/43560</f>
+        <f>F18/43560</f>
         <v/>
       </c>
     </row>
@@ -8709,30 +9733,31 @@
         <v>6</v>
       </c>
       <c r="B22" s="22">
-        <f>120 + 2*3*A22</f>
+        <f>120 + 2*3*A19</f>
         <v/>
       </c>
       <c r="C22" s="20">
-        <f>60 + 2*3*A22</f>
+        <f>60 + 2*3*A19</f>
         <v/>
       </c>
       <c r="D22" s="22">
-        <f>B22 * C22</f>
+        <f>B19 * C19</f>
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>(1/3)*(D21 + D22 + SQRT(D21*D22))</f>
+        <f>(1/3)*(D18 + D19 + SQRT(D18*D19))</f>
         <v/>
       </c>
       <c r="F22" s="20">
-        <f>F21 + E22</f>
+        <f>F18 + E19</f>
         <v/>
       </c>
       <c r="G22" s="20">
-        <f>F22/43560</f>
-        <v/>
-      </c>
-    </row>
+        <f>F19/43560</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
@@ -8849,7 +9874,7 @@
         </is>
       </c>
       <c r="B29" s="19">
-        <f>B26 / (B27 * SQRT(2 * 32.174 * B28))</f>
+        <f>B21 / (B22 * SQRT(2 * 32.174 * B23))</f>
         <v/>
       </c>
       <c r="C29" s="13" t="inlineStr">
@@ -8875,7 +9900,7 @@
         </is>
       </c>
       <c r="B30" s="30">
-        <f>SQRT(4 * B29 / PI()) * 12</f>
+        <f>SQRT(4 * B24 / PI()) * 12</f>
         <v/>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -8901,7 +9926,7 @@
         </is>
       </c>
       <c r="B31" s="31">
-        <f>F22</f>
+        <f>F19</f>
         <v/>
       </c>
       <c r="C31" s="28" t="inlineStr">
@@ -8915,7 +9940,7 @@
         </is>
       </c>
       <c r="E31" s="32">
-        <f>IF(F22&gt;=B11*0.6, "PASS - DETENTION VOLUME ADEQUATE", "FAIL - EXPAND POND")</f>
+        <f>IF(F19&gt;=B9*0.6, "PASS - DETENTION VOLUME ADEQUATE", "FAIL - EXPAND POND")</f>
         <v/>
       </c>
     </row>
@@ -8939,7 +9964,7 @@
         </is>
       </c>
       <c r="E32" s="29">
-        <f>IF(B32&gt;=1.0, "PASS - FREEBOARD COMPLIANT", "FAIL - OVERTOPPING RISK")</f>
+        <f>IF(B27&gt;=1.0, "PASS - FREEBOARD COMPLIANT", "FAIL - OVERTOPPING RISK")</f>
         <v/>
       </c>
     </row>
@@ -9177,6 +10202,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -9213,7 +10239,7 @@
         </is>
       </c>
       <c r="B17" s="22">
-        <f>(B7 * B9) / B8</f>
+        <f>(B5 * B7) / B6</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -9234,7 +10260,7 @@
         </is>
       </c>
       <c r="B18" s="30">
-        <f>SQRT(4 * B17 * B12)</f>
+        <f>SQRT(4 * B13 * B10)</f>
         <v/>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -9255,7 +10281,7 @@
         </is>
       </c>
       <c r="B19" s="37">
-        <f>B10 / B18</f>
+        <f>B8 / B14</f>
         <v/>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -9276,7 +10302,7 @@
         </is>
       </c>
       <c r="B20" s="37">
-        <f>B11 / B18</f>
+        <f>B9 / B14</f>
         <v/>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -9297,7 +10323,7 @@
         </is>
       </c>
       <c r="B21" s="37">
-        <f>4 * B19 * B20 * (1 - 0.33*(B19^2 + B20^2))</f>
+        <f>4 * B15 * B16 * (1 - 0.33*(B15^2 + B16^2))</f>
         <v/>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -9318,7 +10344,7 @@
         </is>
       </c>
       <c r="B22" s="30">
-        <f>(B6 / (4 * B7 * B9 / B8)) * B18^2 * B21</f>
+        <f>(B4 / (4 * B5 * B7 / B6)) * B14^2 * B17</f>
         <v/>
       </c>
       <c r="C22" s="13" t="inlineStr">
@@ -9339,7 +10365,7 @@
         </is>
       </c>
       <c r="B23" s="30">
-        <f>SQRT(B9^2 + 2*B9*B22) - B9</f>
+        <f>SQRT(B7^2 + 2*B7*B18) - B7</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -9353,6 +10379,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
@@ -9420,7 +10447,7 @@
         </is>
       </c>
       <c r="B28" s="27">
-        <f>B13 - B23</f>
+        <f>B11 - B19</f>
         <v/>
       </c>
       <c r="C28" s="28" t="inlineStr">
@@ -9434,7 +10461,7 @@
         </is>
       </c>
       <c r="E28" s="29">
-        <f>IF((B13-B23)&gt;=2.0, "PASS - SHWT SEPARATION MAINTAINED", "FAIL - GROUNDWATER BREAKOUT RISK")</f>
+        <f>IF((B11-B19)&gt;=2.0, "PASS - SHWT SEPARATION MAINTAINED", "FAIL - GROUNDWATER BREAKOUT RISK")</f>
         <v/>
       </c>
     </row>
@@ -9445,7 +10472,7 @@
         </is>
       </c>
       <c r="B29" s="39">
-        <f>(B13 - B23) * 12</f>
+        <f>(B11 - B19) * 12</f>
         <v/>
       </c>
       <c r="C29" s="28" t="inlineStr">
@@ -9459,7 +10486,7 @@
         </is>
       </c>
       <c r="E29" s="41">
-        <f>IF(((B13-B23)*12)&gt;=24.0, "PASS - SHWT &gt;= 24 INCHES", "FAIL - SHWT VIOLATION")</f>
+        <f>IF(((B11-B19)*12)&gt;=24.0, "PASS", "FAIL")</f>
         <v/>
       </c>
     </row>
@@ -9624,7 +10651,7 @@
         </is>
       </c>
       <c r="B10" s="22">
-        <f>B6^2 / (15 * (B8 + B9))</f>
+        <f>B4^2 / (15 * (B6 + B7))</f>
         <v/>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -9665,7 +10692,7 @@
         </is>
       </c>
       <c r="B12" s="30">
-        <f>5729.578 / B11</f>
+        <f>5729.578 / B9</f>
         <v/>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -9686,7 +10713,7 @@
         </is>
       </c>
       <c r="B13" s="33">
-        <f>B11 * TAN(RADIANS(B7 / 2))</f>
+        <f>B9 * TAN(RADIANS(B5 / 2))</f>
         <v/>
       </c>
       <c r="C13" s="13" t="inlineStr">
@@ -9707,7 +10734,7 @@
         </is>
       </c>
       <c r="B14" s="33">
-        <f>(PI() * B11 * B7) / 180</f>
+        <f>(PI() * B9 * B5) / 180</f>
         <v/>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -9728,7 +10755,7 @@
         </is>
       </c>
       <c r="B15" s="30">
-        <f>B11 * (1/COS(RADIANS(B7/2)) - 1)</f>
+        <f>B9 * (1/COS(RADIANS(B5/2)) - 1)</f>
         <v/>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -9749,7 +10776,7 @@
         </is>
       </c>
       <c r="B16" s="30">
-        <f>B11 * (1 - COS(RADIANS(B7/2)))</f>
+        <f>B9 * (1 - COS(RADIANS(B5/2)))</f>
         <v/>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -9763,6 +10790,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -9859,7 +10887,7 @@
         </is>
       </c>
       <c r="B23" s="22">
-        <f>1.47 * B6 * B20</f>
+        <f>1.47 * B4 * B16</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -9880,7 +10908,7 @@
         </is>
       </c>
       <c r="B24" s="22">
-        <f>B6^2 / (30 * (B21/32.174 + B22))</f>
+        <f>B4^2 / (30 * (B17/32.174 + B18))</f>
         <v/>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -9901,7 +10929,7 @@
         </is>
       </c>
       <c r="B25" s="22">
-        <f>B23 + B24</f>
+        <f>B19 + B20</f>
         <v/>
       </c>
       <c r="C25" s="13" t="inlineStr">
@@ -9915,6 +10943,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -9965,7 +10994,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="30">
-        <f>B29 * C29 * D29</f>
+        <f>B24 * C24 * D24</f>
         <v/>
       </c>
     </row>
@@ -9985,7 +11014,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="30">
-        <f>B30 * C30 * D30</f>
+        <f>B25 * C25 * D25</f>
         <v/>
       </c>
     </row>
@@ -10005,7 +11034,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="30">
-        <f>B31 * C31 * D31</f>
+        <f>B26 * C26 * D26</f>
         <v/>
       </c>
     </row>
@@ -10029,7 +11058,7 @@
         </is>
       </c>
       <c r="E32" s="45">
-        <f>E29 + E30 + E31</f>
+        <f>E24 + E25 + E26</f>
         <v/>
       </c>
     </row>
@@ -10181,6 +11210,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -10277,7 +11307,7 @@
         </is>
       </c>
       <c r="B15" s="30">
-        <f>ABS(B14 - B13)</f>
+        <f>ABS(B9 - B10)</f>
         <v/>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -10318,7 +11348,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>B16 * TAN(RADIANS(B15 / 2))</f>
+        <f>B12 * TAN(RADIANS(B11 / 2))</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -10339,7 +11369,7 @@
         </is>
       </c>
       <c r="B18" s="30">
-        <f>B12 - B17</f>
+        <f>B8 - B13</f>
         <v/>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -10360,7 +11390,7 @@
         </is>
       </c>
       <c r="B19" s="30">
-        <f>(PI() * B16 * B15) / 180</f>
+        <f>(PI() * B12 * B11) / 180</f>
         <v/>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -10374,6 +11404,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -10410,11 +11441,11 @@
         </is>
       </c>
       <c r="B23" s="33">
-        <f>B12 * B12</f>
+        <f>B8 * B8</f>
         <v/>
       </c>
       <c r="C23" s="20">
-        <f>B23 / 43560</f>
+        <f>B18 / 43560</f>
         <v/>
       </c>
       <c r="D23" s="34" t="inlineStr">
@@ -10430,11 +11461,11 @@
         </is>
       </c>
       <c r="B24" s="30">
-        <f>B16*B17 - 0.5*B16^2*RADIANS(B15)</f>
+        <f>B12*B13 - 0.5*B12^2*RADIANS(B11)</f>
         <v/>
       </c>
       <c r="C24" s="20">
-        <f>B24 / 43560</f>
+        <f>B19 / 43560</f>
         <v/>
       </c>
       <c r="D24" s="14" t="inlineStr">
@@ -10450,11 +11481,11 @@
         </is>
       </c>
       <c r="B25" s="48">
-        <f>B23 - B24</f>
+        <f>B18 - B19</f>
         <v/>
       </c>
       <c r="C25" s="25">
-        <f>B25 / 43560</f>
+        <f>B20 / 43560</f>
         <v/>
       </c>
       <c r="D25" s="49" t="inlineStr">
@@ -10604,7 +11635,7 @@
         </is>
       </c>
       <c r="B9" s="37">
-        <f>(PI()/4) * (B6/12)^2</f>
+        <f>(PI()/4) * (B4/12)^2</f>
         <v/>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -10625,7 +11656,7 @@
         </is>
       </c>
       <c r="B10" s="37">
-        <f>(B6/12) / 4</f>
+        <f>(B4/12) / 4</f>
         <v/>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -10646,7 +11677,7 @@
         </is>
       </c>
       <c r="B11" s="30">
-        <f>(1.486 / B7) * B10^(2/3) * SQRT(B8)</f>
+        <f>(1.486 / B5) * B8^(2/3) * SQRT(B6)</f>
         <v/>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -10667,7 +11698,7 @@
         </is>
       </c>
       <c r="B12" s="22">
-        <f>B11 * B9 * 448.83</f>
+        <f>B9 * B7 * 448.83</f>
         <v/>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -10688,7 +11719,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>B11</f>
+        <f>B9</f>
         <v/>
       </c>
       <c r="C13" s="28" t="inlineStr">
@@ -10702,10 +11733,11 @@
         </is>
       </c>
       <c r="E13" s="29">
-        <f>IF(B11&gt;=2.0, "PASS - SCOURING VELOCITY MAINTAINED", "FAIL - SLUGGING RISK")</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(B9&gt;=2.0, "PASS - SCOURING VELOCITY MAINTAINED", "FAIL - SLUGGING RISK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -10802,7 +11834,7 @@
         </is>
       </c>
       <c r="B20" s="22">
-        <f>(B19 * B18) / 4</f>
+        <f>(B15 * B14) / 4</f>
         <v/>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -10823,7 +11855,7 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>B20 / 7.48052</f>
+        <f>B16 / 7.48052</f>
         <v/>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -10864,7 +11896,7 @@
         </is>
       </c>
       <c r="B23" s="30">
-        <f>(PI()/4) * B22^2</f>
+        <f>(PI()/4) * B18^2</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -10885,7 +11917,7 @@
         </is>
       </c>
       <c r="B24" s="30">
-        <f>B21 / B23</f>
+        <f>B17 / B19</f>
         <v/>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -10899,6 +11931,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -11015,7 +12048,7 @@
         </is>
       </c>
       <c r="B32" s="30">
-        <f>(B18 / 448.83) / ((PI()/4)*(B28/12)^2)</f>
+        <f>(B14 / 448.83) / ((PI()/4)*(B22/12)^2)</f>
         <v/>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -11036,7 +12069,7 @@
         </is>
       </c>
       <c r="B33" s="30">
-        <f>10.44 * B29 * B18^1.852 / (B30^1.852 * B28^4.87)</f>
+        <f>10.44 * B23 * B14^1.852 / (B24^1.852 * B22^4.87)</f>
         <v/>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -11057,7 +12090,7 @@
         </is>
       </c>
       <c r="B34" s="30">
-        <f>0.10 * B33</f>
+        <f>0.10 * B27</f>
         <v/>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -11078,7 +12111,7 @@
         </is>
       </c>
       <c r="B35" s="30">
-        <f>B31 + B33 + B34</f>
+        <f>B25 + B27 + B28</f>
         <v/>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -11119,7 +12152,7 @@
         </is>
       </c>
       <c r="B37" s="30">
-        <f>(B18 * B35) / (3960 * B36)</f>
+        <f>(B14 * B29) / (3960 * B30)</f>
         <v/>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -11140,7 +12173,7 @@
         </is>
       </c>
       <c r="B38" s="52">
-        <f>ROUNDUP(B37 * 1.15, 0)</f>
+        <f>ROUNDUP(B31 * 1.15, 0)</f>
         <v/>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -11295,7 +12328,7 @@
         </is>
       </c>
       <c r="B9" s="30">
-        <f>135 / (B8 + 18)^0.82</f>
+        <f>135 / (B6 + 18)^0.82</f>
         <v/>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -11316,7 +12349,7 @@
         </is>
       </c>
       <c r="B10" s="33">
-        <f>B6 * B7 * B9</f>
+        <f>B4 * B5 * B7</f>
         <v/>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -11330,6 +12363,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -11426,7 +12460,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>((B10 * B16) / (0.56 * B15^(5/3) * B14^0.5))^(3/8)</f>
+        <f>( (B8 * B13) / (0.56 * B12^(5/3) * B11^0.5) )^(3/8)</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -11460,10 +12494,11 @@
         </is>
       </c>
       <c r="E18" s="29">
-        <f>IF(B17&lt;=B18, "PASS - GUTTER SPREAD WITHIN SHOULDER", "FAIL - TRAFFIC LANE INUNDATED")</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(B14&lt;=B15, "PASS - GUTTER SPREAD WITHIN SHOULDER", "FAIL - TRAFFIC LANE INUNDATED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -11580,7 +12615,7 @@
         </is>
       </c>
       <c r="B26" s="30">
-        <f>(B22/12) * (1.0 + 0.038 * (B10 / ((PI()/4)*(B22/12)^2 * SQRT(B22/12)))^1.5)</f>
+        <f>(B18/12) * ( 1.0 + 0.038 * (B8 / ((PI()/4)*(B18/12)^2 * SQRT(B18/12)))^1.5 )</f>
         <v/>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -11601,7 +12636,7 @@
         </is>
       </c>
       <c r="B27" s="30">
-        <f>2.5 + (1 + 0.5 + 29*B25^2*B23/((B22/12)^(4/3))) * ((B10/((PI()/4)*(B22/12)^2))^2 / (2*32.174)) - B24*B23</f>
+        <f>2.5 + (1 + 0.5 + 29*B21^2*B19/((B18/12)^(4/3))) * ((B8/((PI()/4)*(B18/12)^2))^2 / (2*32.174)) - B19*B20</f>
         <v/>
       </c>
       <c r="C27" s="13" t="inlineStr">
@@ -11622,7 +12657,7 @@
         </is>
       </c>
       <c r="B28" s="30">
-        <f>MAX(B26, B27)</f>
+        <f>MAX(B22, B23)</f>
         <v/>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -11683,7 +12718,7 @@
         </is>
       </c>
       <c r="B31" s="27">
-        <f>B29 - (B30 + B28)</f>
+        <f>B25 - (B26 + B24)</f>
         <v/>
       </c>
       <c r="C31" s="28" t="inlineStr">
@@ -11697,7 +12732,7 @@
         </is>
       </c>
       <c r="E31" s="29">
-        <f>IF((B29-(B30+B28))&gt;=1.0, "PASS - FREEBOARD &gt;= 1.0 FT", "FAIL - ROADWAY OVERTOPPING RISK")</f>
+        <f>IF((B25-(B26+B24))&gt;=1.0, "PASS - FREEBOARD &gt;= 1.0 FT", "FAIL - ROADWAY OVERTOPPING RISK")</f>
         <v/>
       </c>
     </row>
@@ -11955,6 +12990,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -11991,7 +13027,7 @@
         </is>
       </c>
       <c r="B18" s="30">
-        <f>4 * B6</f>
+        <f>4 * B4</f>
         <v/>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -12012,7 +13048,7 @@
         </is>
       </c>
       <c r="B19" s="30">
-        <f>B6 * B6</f>
+        <f>B4 * B4</f>
         <v/>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -12033,7 +13069,7 @@
         </is>
       </c>
       <c r="B20" s="22">
-        <f>B10 * B9 * B18 * B8</f>
+        <f>B8 * B7 * B13 * B6</f>
         <v/>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -12054,7 +13090,7 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>(1 - SIN(RADIANS(B12))) * TAN(RADIANS(0.75*B12)) * B13 * B18 * B11</f>
+        <f>(1 - SIN(RADIANS(B10))) * TAN(RADIANS(0.75*B10)) * B11 * B13 * B9</f>
         <v/>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -12075,7 +13111,7 @@
         </is>
       </c>
       <c r="B22" s="30">
-        <f>(B20 + B21) / 1000</f>
+        <f>(B15 + B16) / 1000</f>
         <v/>
       </c>
       <c r="C22" s="13" t="inlineStr">
@@ -12096,7 +13132,7 @@
         </is>
       </c>
       <c r="B23" s="30">
-        <f>(B13 * B14 * B19) / 1000</f>
+        <f>(B11 * B12 * B14) / 1000</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -12117,7 +13153,7 @@
         </is>
       </c>
       <c r="B24" s="45">
-        <f>B22 + B23</f>
+        <f>B17 + B18</f>
         <v/>
       </c>
       <c r="C24" s="54" t="inlineStr">
@@ -12138,7 +13174,7 @@
         </is>
       </c>
       <c r="B25" s="30">
-        <f>B24 / 2.5</f>
+        <f>B19 / 2.5</f>
         <v/>
       </c>
       <c r="C25" s="13" t="inlineStr">
@@ -12159,7 +13195,7 @@
         </is>
       </c>
       <c r="B26" s="30">
-        <f>B25 / 2.0</f>
+        <f>B20 / 2.0</f>
         <v/>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -12173,6 +13209,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -12269,7 +13306,7 @@
         </is>
       </c>
       <c r="B33" s="37">
-        <f>1 - (DEGREES(ATAN(B6 / B32)) / 90) * (((B31-1)*B30 + (B30-1)*B31) / (B30 * B31))</f>
+        <f>1 - (DEGREES(ATAN(B4 / B26)) / 90) * (((B24-1)*B25 + (B25-1)*B24) / (B24 * B25))</f>
         <v/>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -12290,7 +13327,7 @@
         </is>
       </c>
       <c r="B34" s="22">
-        <f>B30 * B31 * B25 * B33</f>
+        <f>B24 * B25 * B20 * B27</f>
         <v/>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -12311,7 +13348,7 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>B34 / 2.0</f>
+        <f>B28 / 2.0</f>
         <v/>
       </c>
       <c r="C35" s="54" t="inlineStr">

</xml_diff>

<commit_message>
feat(periodic-table): add interactive periodic table, cation-anion balancer, radicals reference, and fix element grid alignment
</commit_message>
<xml_diff>
--- a/public/Civil_Engineering_Master_Toolbox.xlsx
+++ b/public/Civil_Engineering_Master_Toolbox.xlsx
@@ -28,6 +28,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NPSH &amp; Pump Cavitation" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stormwater &amp; TR-55 CN" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidation &amp; Surcharge" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Periodic Table &amp; Chemistry" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -150,7 +151,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -186,11 +187,55 @@
         <color rgb="000F172A"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -387,6 +432,14 @@
     <xf numFmtId="164" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -752,7 +805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -782,7 +835,7 @@
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1. WORKBOOK NAVIGATION &amp; MODULE DIRECTORY (21 WORKSHEETS)</t>
+          <t>1. WORKBOOK NAVIGATION &amp; MODULE DIRECTORY (22 WORKSHEETS)</t>
         </is>
       </c>
     </row>
@@ -1248,185 +1301,231 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Periodic Table &amp; Chemistry</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Water Chemistry &amp; Treatment</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>NCEES § 6.1 • Periodic Table &amp; Radicals</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>118 elements, atomic weights, common water treatment radicals, equivalent weights EW = MW/|z|, Problem #92 cation-anion balance solver &amp; stoichiometric ratios</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>2. STANDARDIZED COLOR CODING &amp; CELL CONVENTIONS</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>User Modifiable Input Parameter</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Soft Blue fill (#EFF6FF) with thin border. Modify these values to customize scenarios.</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="C29" s="72" t="n"/>
+      <c r="D29" s="73" t="n"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Live Dynamic Excel Formula</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>White / Neutral cell containing real formulas (=SUM, =IF, =SQRT, etc.). Do not overwrite.</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="C30" s="72" t="n"/>
+      <c r="D30" s="73" t="n"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Code Check / Design Status: PASS</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Soft Green fill (#DCFCE7) indicating compliance with NCEES, ACI, AASHTO, or OSHA criteria.</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="C31" s="72" t="n"/>
+      <c r="D31" s="73" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Code Check / Design Status: FAIL</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Soft Red fill (#FEE2E2) indicating safety factor violation or overtopping hazard.</t>
         </is>
       </c>
-    </row>
-    <row r="32"/>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="C32" s="72" t="n"/>
+      <c r="D32" s="73" t="n"/>
+    </row>
+    <row r="33"/>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>3. NCEES CIVIL PE FREQUENT UNIT CONVERSIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>1 acre-foot</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>43,560 ft³ = 325,851 gallons</t>
         </is>
       </c>
     </row>
     <row r="35" ht="19" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>1 ft³ of Water</t>
+          <t>1 acre-foot</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>7.48052 gallons = 62.4 lbs (at 60°F)</t>
-        </is>
-      </c>
+          <t>43,560 ft³ = 325,851 gallons</t>
+        </is>
+      </c>
+      <c r="C35" s="72" t="n"/>
+      <c r="D35" s="73" t="n"/>
     </row>
     <row r="36" ht="19" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>1 cubic foot per second (cfs)</t>
+          <t>1 ft³ of Water</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>448.83 gallons per minute (gpm) = 0.6463 MGD</t>
-        </is>
-      </c>
+          <t>7.48052 gallons = 62.4 lbs (at 60°F)</t>
+        </is>
+      </c>
+      <c r="C36" s="72" t="n"/>
+      <c r="D36" s="73" t="n"/>
     </row>
     <row r="37" ht="19" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>1 psi pressure head</t>
+          <t>1 cubic foot per second (cfs)</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>2.307 feet of water column (ft H₂O)</t>
-        </is>
-      </c>
+          <t>448.83 gallons per minute (gpm) = 0.6463 MGD</t>
+        </is>
+      </c>
+      <c r="C37" s="72" t="n"/>
+      <c r="D37" s="73" t="n"/>
     </row>
     <row r="38" ht="19" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Standard Atmospheric Pressure (Sea Level)</t>
+          <t>1 psi pressure head</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>14.696 psia = 2,116 psf = 33.90 ft H₂O = 29.92 in Hg</t>
-        </is>
-      </c>
+          <t>2.307 feet of water column (ft H₂O)</t>
+        </is>
+      </c>
+      <c r="C38" s="72" t="n"/>
+      <c r="D38" s="73" t="n"/>
     </row>
     <row r="39" ht="19" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Acceleration of Gravity (g)</t>
+          <t>Standard Atmospheric Pressure (Sea Level)</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>32.174 ft/s² = 9.80665 m/s²</t>
-        </is>
-      </c>
+          <t>14.696 psia = 2,116 psf = 33.90 ft H₂O = 29.92 in Hg</t>
+        </is>
+      </c>
+      <c r="C39" s="72" t="n"/>
+      <c r="D39" s="73" t="n"/>
     </row>
     <row r="40" ht="19" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Density of Normal-Weight Concrete</t>
+          <t>Acceleration of Gravity (g)</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>145 to 150 lbs/ft³ (pcf)</t>
-        </is>
-      </c>
+          <t>32.174 ft/s² = 9.80665 m/s²</t>
+        </is>
+      </c>
+      <c r="C40" s="72" t="n"/>
+      <c r="D40" s="73" t="n"/>
     </row>
     <row r="41" ht="19" customHeight="1">
       <c r="A41" s="10" t="inlineStr">
         <is>
+          <t>Density of Normal-Weight Concrete</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>145 to 150 lbs/ft³ (pcf)</t>
+        </is>
+      </c>
+      <c r="C41" s="72" t="n"/>
+      <c r="D41" s="73" t="n"/>
+    </row>
+    <row r="42" ht="19" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
           <t>Modulus of Elasticity of Steel (Es)</t>
         </is>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>29,000,000 psi (29,000 ksi)</t>
         </is>
       </c>
+      <c r="C42" s="72" t="n"/>
+      <c r="D42" s="73" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B42:D42"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B37:D37"/>
-    <mergeCell ref="A27:G27"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A4:G4"/>
     <mergeCell ref="B35:D35"/>
-    <mergeCell ref="A4:G4"/>
     <mergeCell ref="B40:D40"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B39:D39"/>
-    <mergeCell ref="A33:G33"/>
     <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="A28:G28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6912,11 +7011,11 @@
         </is>
       </c>
       <c r="B20" s="19">
-        <f>(1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5)))</f>
+        <f>(1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7)))</f>
         <v/>
       </c>
       <c r="C20" s="20">
-        <f>ROUND((1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5))), 4)</f>
+        <f>ROUND((1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7))), 4)</f>
         <v/>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -6937,19 +7036,19 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>0.5 * B6 * B4^2 * C18</f>
+        <f>0.5 * B8 * B6^2 * B20</f>
         <v/>
       </c>
       <c r="C21" s="20">
-        <f>0.5 * B6 * B4^2 * ((1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5))))</f>
+        <f>0.5 * B8 * B6^2 * ((1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7))))</f>
         <v/>
       </c>
       <c r="D21" s="22">
-        <f>B4 / 3</f>
+        <f>B6 / 3</f>
         <v/>
       </c>
       <c r="E21" s="22">
-        <f>C19 * D19</f>
+        <f>C21 * D21</f>
         <v/>
       </c>
     </row>
@@ -6960,19 +7059,19 @@
         </is>
       </c>
       <c r="B22" s="22">
-        <f>B11 * B4 * C18</f>
+        <f>B13 * B6 * B20</f>
         <v/>
       </c>
       <c r="C22" s="20">
-        <f>B11 * B4 * ((1-SIN(RADIANS(B5)))/(1+SIN(RADIANS(B5))))</f>
+        <f>B13 * B6 * ((1-SIN(RADIANS(B7)))/(1+SIN(RADIANS(B7))))</f>
         <v/>
       </c>
       <c r="D22" s="22">
-        <f>B4 / 2</f>
+        <f>B6 / 2</f>
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>C20 * D20</f>
+        <f>C22 * D22</f>
         <v/>
       </c>
     </row>
@@ -6988,7 +7087,7 @@
         </is>
       </c>
       <c r="C23" s="25">
-        <f>C19 + C20</f>
+        <f>C21 + C22</f>
         <v/>
       </c>
       <c r="D23" s="24" t="inlineStr">
@@ -6997,7 +7096,7 @@
         </is>
       </c>
       <c r="E23" s="26">
-        <f>E19 + E20</f>
+        <f>E21 + E22</f>
         <v/>
       </c>
     </row>
@@ -7043,19 +7142,19 @@
         </is>
       </c>
       <c r="B27" s="22">
-        <f>(B4 - B8) * B9 * B12</f>
+        <f>(B6 - B10) * B11 * B14</f>
         <v/>
       </c>
       <c r="C27" s="20">
-        <f>(B4 - B8) * B9 * B12</f>
+        <f>(B6 - B10) * B11 * B14</f>
         <v/>
       </c>
       <c r="D27" s="22">
-        <f>B10 + B9/2</f>
+        <f>B12 + B11/2</f>
         <v/>
       </c>
       <c r="E27" s="22">
-        <f>C24 * D24</f>
+        <f>C27 * D27</f>
         <v/>
       </c>
     </row>
@@ -7066,19 +7165,19 @@
         </is>
       </c>
       <c r="B28" s="22">
-        <f>B7 * B8 * B12</f>
+        <f>B9 * B10 * B14</f>
         <v/>
       </c>
       <c r="C28" s="20">
-        <f>B7 * B8 * B12</f>
+        <f>B9 * B10 * B14</f>
         <v/>
       </c>
       <c r="D28" s="22">
-        <f>B7 / 2</f>
+        <f>B9 / 2</f>
         <v/>
       </c>
       <c r="E28" s="22">
-        <f>C25 * D25</f>
+        <f>C28 * D28</f>
         <v/>
       </c>
     </row>
@@ -7089,19 +7188,19 @@
         </is>
       </c>
       <c r="B29" s="22">
-        <f>(B7 - B10 - B9) * (B4 - B8) * B6</f>
+        <f>(B9 - B12 - B11) * (B6 - B10) * B8</f>
         <v/>
       </c>
       <c r="C29" s="20">
-        <f>(B7 - B10 - B9) * (B4 - B8) * B6</f>
+        <f>(B9 - B12 - B11) * (B6 - B10) * B8</f>
         <v/>
       </c>
       <c r="D29" s="22">
-        <f>B7 - (B7 - B10 - B9)/2</f>
+        <f>B9 - (B9 - B12 - B11)/2</f>
         <v/>
       </c>
       <c r="E29" s="22">
-        <f>C26 * D26</f>
+        <f>C29 * D29</f>
         <v/>
       </c>
     </row>
@@ -7117,7 +7216,7 @@
         </is>
       </c>
       <c r="C30" s="25">
-        <f>C24 + C25 + C26</f>
+        <f>C27 + C28 + C29</f>
         <v/>
       </c>
       <c r="D30" s="24" t="inlineStr">
@@ -7126,7 +7225,7 @@
         </is>
       </c>
       <c r="E30" s="26">
-        <f>E24 + E25 + E26</f>
+        <f>E27 + E28 + E29</f>
         <v/>
       </c>
     </row>
@@ -7172,7 +7271,7 @@
         </is>
       </c>
       <c r="B34" s="27">
-        <f>E27 / E21</f>
+        <f>E30 / E23</f>
         <v/>
       </c>
       <c r="C34" s="28" t="inlineStr">
@@ -7181,11 +7280,11 @@
         </is>
       </c>
       <c r="D34" s="29">
-        <f>E27 / E21</f>
+        <f>E30 / E23</f>
         <v/>
       </c>
       <c r="E34" s="29">
-        <f>IF(B30&gt;=2.0, "PASS - OVERTURNING SAFE", "FAIL - UNDERSIZED TOE")</f>
+        <f>IF(B34&gt;=2.0, "PASS - OVERTURNING SAFE", "FAIL - UNDERSIZED TOE")</f>
         <v/>
       </c>
     </row>
@@ -7196,7 +7295,7 @@
         </is>
       </c>
       <c r="B35" s="27">
-        <f>(C27 * B13) / C21</f>
+        <f>(C30 * B15) / C23</f>
         <v/>
       </c>
       <c r="C35" s="28" t="inlineStr">
@@ -7205,11 +7304,11 @@
         </is>
       </c>
       <c r="D35" s="29">
-        <f>(C27 * B13) / C21</f>
+        <f>(C30 * B15) / C23</f>
         <v/>
       </c>
       <c r="E35" s="29">
-        <f>IF(B31&gt;=1.5, "PASS - SLIDING SAFE", "FAIL - ADD SHEAR KEY")</f>
+        <f>IF(B35&gt;=1.5, "PASS - SLIDING SAFE", "FAIL - ADD SHEAR KEY")</f>
         <v/>
       </c>
     </row>
@@ -7220,7 +7319,7 @@
         </is>
       </c>
       <c r="B36" s="30">
-        <f>(E27 - E21) / C27</f>
+        <f>(E30 - E23) / C30</f>
         <v/>
       </c>
       <c r="C36" s="13" t="inlineStr">
@@ -7228,10 +7327,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr">
-        <is>
-          <t>x_bar = (M_r - M_ot) / W</t>
-        </is>
+      <c r="D36" s="14">
+        <f>(E30 - E23) / C30</f>
+        <v/>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
@@ -7246,7 +7344,7 @@
         </is>
       </c>
       <c r="B37" s="27">
-        <f>ABS(B7/2 - B32)</f>
+        <f>ABS(B9/2 - B36)</f>
         <v/>
       </c>
       <c r="C37" s="28" t="inlineStr">
@@ -7255,11 +7353,11 @@
         </is>
       </c>
       <c r="D37" s="29">
-        <f>B7/6</f>
+        <f>B9/6</f>
         <v/>
       </c>
       <c r="E37" s="29">
-        <f>IF(B33&lt;=(B7/6), "PASS - WITHIN MIDDLE THIRD (KERN)", "FAIL - TENSION AT HEEL")</f>
+        <f>IF(B37&lt;=(B9/6), "PASS - WITHIN MIDDLE THIRD (KERN)", "FAIL - TENSION AT HEEL")</f>
         <v/>
       </c>
     </row>
@@ -7270,7 +7368,7 @@
         </is>
       </c>
       <c r="B38" s="31">
-        <f>(C27 / B7) * (1 + 6*B33/B7)</f>
+        <f>(C30 / B9) * (1 + 6*B37/B9)</f>
         <v/>
       </c>
       <c r="C38" s="28" t="inlineStr">
@@ -7279,11 +7377,11 @@
         </is>
       </c>
       <c r="D38" s="32">
-        <f>B14 - B34</f>
+        <f>B16 - B38</f>
         <v/>
       </c>
       <c r="E38" s="32">
-        <f>IF(B34&lt;=B14, "PASS - BEARING CAPACITY ADEQUATE", "FAIL - EXCEEDS BEARING CAPACITY")</f>
+        <f>IF(B38&lt;=B16, "PASS - BEARING CAPACITY ADEQUATE", "FAIL - EXCEEDS BEARING CAPACITY")</f>
         <v/>
       </c>
     </row>
@@ -7469,10 +7567,9 @@
           <t>COMPOSITE CURVE NUMBER (CN)</t>
         </is>
       </c>
-      <c r="B10" s="68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B10" s="68">
+        <f>(B6*0.25 + B7*0.35 + B8*0.25 + B9*0.15)</f>
+        <v/>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
@@ -7480,7 +7577,7 @@
         </is>
       </c>
       <c r="D10" s="69">
-        <f>SUM(D4:D7)</f>
+        <f>SUM(D6:D7)</f>
         <v/>
       </c>
       <c r="E10" s="68" t="inlineStr">
@@ -9238,7 +9335,7 @@
           <t>Target = 0.00 inches (Fully dissipated)</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr">
+      <c r="E55" s="70" t="inlineStr">
         <is>
           <t>PASS - SETTLEMENT ELIMINATED</t>
         </is>
@@ -9304,6 +9401,1596 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A41:G41"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="74" customWidth="1" min="1" max="1"/>
+    <col width="119" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="74" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SOLVEDIN6 CIVIL MASTER TOOLBOX - TAB 22: PERIODIC TABLE &amp; WATER CHEMISTRY LAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NCEES PE Reference Handbook § 6.1 • Periodic Table, Equivalent Weights &amp; Problem #92 Cation-Anion Balance Solver</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1. COMMON NCEES WATER &amp; ENVIRONMENTAL ELEMENTS &amp; ATOMIC WEIGHTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Element Name</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Atomic No. (Z)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Atomic Weight (g/mol)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Common Valence</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Primary Environmental Engineering Application</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Hydrogen</t>
+        </is>
+      </c>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="37" t="n">
+        <v>1.008</v>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>pH definition, acid-base equilibrium, hydration reactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>12.011</v>
+      </c>
+      <c r="E7" s="38" t="inlineStr">
+        <is>
+          <t>+4, -4</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Carbonate equilibrium, alkalinity, BOD/COD organic carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Nitrogen</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>14.007</v>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>-3 to +5</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Nutrient, Ammonia, Nitrite, Nitrate (MCL = 10 mg/L as N), TKN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Oxygen</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="37" t="n">
+        <v>15.999</v>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>-2</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Dissolved oxygen (DO), oxidation-reduction, aeration, ozone</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Sodium</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>Na</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="D10" s="37" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Major cation, Sodium Adsorption Ratio (SAR), ion exchange</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Magnesium</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" s="37" t="n">
+        <v>24.305</v>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Secondary hardness contributor, excess lime softening precipitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Aluminum</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" s="37" t="n">
+        <v>26.982</v>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Coagulation with alum [Al2(SO4)3·14H2O], sweep flocculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Phosphorus</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" s="37" t="n">
+        <v>30.974</v>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>+5</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Limiting nutrient, orthophosphate, biological phosphorus removal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Sulfur</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" s="37" t="n">
+        <v>32.06</v>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>-2 to +6</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Sulfate salinity, hydrogen sulfide odor/corrosion, acid mine drainage</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Chlorine</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="D15" s="37" t="n">
+        <v>35.453</v>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Disinfection (free/combined chlorine), chloride salinity, CT credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Potassium</t>
+        </is>
+      </c>
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="D16" s="37" t="n">
+        <v>39.098</v>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Agricultural runoff nutrient, major intracellular cation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Calcium</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="37" t="n">
+        <v>40.078</v>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Primary water hardness cation, lime softening [Ca(OH)2], scaling</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Iron</t>
+        </is>
+      </c>
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>Fe</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="D18" s="37" t="n">
+        <v>55.845</v>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>+2, +3</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Ferric chloride coagulant, red water aesthetic secondary MCL (0.3 mg/L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Copper</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>Cu</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="n">
+        <v>29</v>
+      </c>
+      <c r="D19" s="37" t="n">
+        <v>63.546</v>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>+1, +2</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Lead and Copper Rule (Action Level = 1.3 mg/L), pipe corrosion</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Arsenic</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>As</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="D20" s="37" t="n">
+        <v>74.922</v>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>+3, +5</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Toxic carcinogen, Primary MCL = 0.010 mg/L, arsenite vs arsenate</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>Pb</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="n">
+        <v>82</v>
+      </c>
+      <c r="D21" s="37" t="n">
+        <v>207.2</v>
+      </c>
+      <c r="E21" s="38" t="inlineStr">
+        <is>
+          <t>+2, +4</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Toxic neurotoxin, Lead and Copper Rule (Action Level = 0.015 mg/L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2. COMMON WATER TREATMENT RADICALS &amp; EQUIVALENT WEIGHTS (EW = MW / |z|)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Radical / Chemical Formula</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Common Radical Name</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Molecular Weight (g/mol)</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Absolute Valence |z|</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Equivalent Weight (g/eq)</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Water Treatment &amp; Chemistry Function</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>H⁺</t>
+        </is>
+      </c>
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>Hydrogen Ion</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>1.008</v>
+      </c>
+      <c r="D25" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="37">
+        <f>C25 / D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Acidity, hydronium ion activity, pH = -log10[H+]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>OH⁻</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>Hydroxide</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="n">
+        <v>17.007</v>
+      </c>
+      <c r="D26" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="37">
+        <f>C26 / D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>Basicity, caustic soda NaOH, lime softening precipitant</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Ca²⁺</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>Calcium Cation</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>40.078</v>
+      </c>
+      <c r="D27" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="37">
+        <f>C27 / D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Hardness, CaCO3 precipitation at pH ~9.3 in softening</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Mg²⁺</t>
+        </is>
+      </c>
+      <c r="B28" s="38" t="inlineStr">
+        <is>
+          <t>Magnesium Cation</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="n">
+        <v>24.305</v>
+      </c>
+      <c r="D28" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="37">
+        <f>C28 / D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Hardness, Mg(OH)2 precipitation at pH ~10.8 (excess lime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Na⁺</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>Sodium Cation</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="D29" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="37">
+        <f>C29 / D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Soluble monovalent cation, cation-exchange softening regenerant</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>HCO₃⁻</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>Bicarbonate</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="n">
+        <v>61.017</v>
+      </c>
+      <c r="D30" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="37">
+        <f>C30 / D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Natural alkalinity buffer in pH range 4.5 to 8.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>CO₃²⁻</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>Carbonate</t>
+        </is>
+      </c>
+      <c r="C31" s="20" t="n">
+        <v>60.009</v>
+      </c>
+      <c r="D31" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="37">
+        <f>C31 / D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>High-pH alkalinity buffer, soda ash (Na2CO3) addition</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>SO₄²⁻</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>Sulfate</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="n">
+        <v>96.06399999999999</v>
+      </c>
+      <c r="D32" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="37">
+        <f>C32 / D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>Non-carbonate hardness counter-ion, alum coagulation byproduct</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Cl⁻</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>Chloride</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="n">
+        <v>35.453</v>
+      </c>
+      <c r="D33" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="37">
+        <f>C33 / D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Conservative tracer, saline intrusion, secondary MCL = 250 mg/L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>NO₃⁻</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>Nitrate</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="n">
+        <v>62.005</v>
+      </c>
+      <c r="D34" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="37">
+        <f>C34 / D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Methemoglobinemia contaminant, primary MCL = 10 mg/L as N</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>PO₄³⁻</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>Orthophosphate</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="n">
+        <v>94.971</v>
+      </c>
+      <c r="D35" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" s="37">
+        <f>C35 / D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Nutrient, lead/copper corrosion inhibitor film former</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>CaCO₃</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>Calcium Carbonate</t>
+        </is>
+      </c>
+      <c r="C36" s="20" t="n">
+        <v>100.087</v>
+      </c>
+      <c r="D36" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="37">
+        <f>C36 / D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Standard universal basis for hardness &amp; alkalinity (EW = 50.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>3. CATION-ANION CHARGE BALANCE SOLVER (PROBLEM #92 LIVE EXAM CASE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Water Quality Ion Parameter</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Measured Conc. (mg/L)</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Valence |z|</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Formula Weight (g/mol)</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Equivalent Wt (mg/meq)</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Normality (meq/L)</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Ion Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Calcium (Ca²⁺)</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n">
+        <v>40.08</v>
+      </c>
+      <c r="C40" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="30" t="n">
+        <v>40.078</v>
+      </c>
+      <c r="E40" s="30">
+        <f>D40 / C40</f>
+        <v/>
+      </c>
+      <c r="F40" s="20">
+        <f>B40 / E40</f>
+        <v/>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>Cation (+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>Magnesium (Mg²⁺)</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="n">
+        <v>24.31</v>
+      </c>
+      <c r="C41" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="30" t="n">
+        <v>24.305</v>
+      </c>
+      <c r="E41" s="30">
+        <f>D41 / C41</f>
+        <v/>
+      </c>
+      <c r="F41" s="20">
+        <f>B41 / E41</f>
+        <v/>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>Cation (+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>Sodium (Na⁺)</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="30" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="E42" s="30">
+        <f>D42 / C42</f>
+        <v/>
+      </c>
+      <c r="F42" s="20">
+        <f>B42 / E42</f>
+        <v/>
+      </c>
+      <c r="G42" s="13" t="inlineStr">
+        <is>
+          <t>Cation (+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>Potassium (K⁺)</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="30" t="n">
+        <v>39.098</v>
+      </c>
+      <c r="E43" s="30">
+        <f>D43 / C43</f>
+        <v/>
+      </c>
+      <c r="F43" s="20">
+        <f>B43 / E43</f>
+        <v/>
+      </c>
+      <c r="G43" s="13" t="inlineStr">
+        <is>
+          <t>Cation (+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>TOTAL MEASURED CATIONS (Σ Cations)</t>
+        </is>
+      </c>
+      <c r="B44" s="45">
+        <f>SUM(F40:F43)</f>
+        <v/>
+      </c>
+      <c r="C44" s="54" t="inlineStr">
+        <is>
+          <t>meq/L</t>
+        </is>
+      </c>
+      <c r="D44" s="44" t="inlineStr">
+        <is>
+          <t>Σ (mg/L / EW) for all cations</t>
+        </is>
+      </c>
+      <c r="E44" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F44" s="25">
+        <f>B44</f>
+        <v/>
+      </c>
+      <c r="G44" s="54" t="inlineStr">
+        <is>
+          <t>Total Cations</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Bicarbonate (HCO₃⁻)</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="n">
+        <v>183</v>
+      </c>
+      <c r="C45" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="30" t="n">
+        <v>61.017</v>
+      </c>
+      <c r="E45" s="30">
+        <f>D45 / C45</f>
+        <v/>
+      </c>
+      <c r="F45" s="20">
+        <f>B45 / E45</f>
+        <v/>
+      </c>
+      <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>Anion (-)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>Sulfate (SO₄²⁻)</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="n">
+        <v>96.06</v>
+      </c>
+      <c r="C46" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" s="30" t="n">
+        <v>96.06399999999999</v>
+      </c>
+      <c r="E46" s="30">
+        <f>D46 / C46</f>
+        <v/>
+      </c>
+      <c r="F46" s="20">
+        <f>B46 / E46</f>
+        <v/>
+      </c>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>Anion (-)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>Chloride (Cl⁻)</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="n">
+        <v>35.45</v>
+      </c>
+      <c r="C47" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="30" t="n">
+        <v>35.453</v>
+      </c>
+      <c r="E47" s="30">
+        <f>D47 / C47</f>
+        <v/>
+      </c>
+      <c r="F47" s="20">
+        <f>B47 / E47</f>
+        <v/>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t>Anion (-)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Nitrate (NO₃⁻)</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="30" t="n">
+        <v>62.005</v>
+      </c>
+      <c r="E48" s="30">
+        <f>D48 / C48</f>
+        <v/>
+      </c>
+      <c r="F48" s="20">
+        <f>B48 / E48</f>
+        <v/>
+      </c>
+      <c r="G48" s="13" t="inlineStr">
+        <is>
+          <t>Anion (-)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="23" t="inlineStr">
+        <is>
+          <t>TOTAL MEASURED ANIONS (Σ Anions)</t>
+        </is>
+      </c>
+      <c r="B49" s="45">
+        <f>SUM(F45:F48)</f>
+        <v/>
+      </c>
+      <c r="C49" s="54" t="inlineStr">
+        <is>
+          <t>meq/L</t>
+        </is>
+      </c>
+      <c r="D49" s="44" t="inlineStr">
+        <is>
+          <t>Σ (mg/L / EW) for all anions</t>
+        </is>
+      </c>
+      <c r="E49" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F49" s="25">
+        <f>B49</f>
+        <v/>
+      </c>
+      <c r="G49" s="54" t="inlineStr">
+        <is>
+          <t>Total Anions</t>
+        </is>
+      </c>
+    </row>
+    <row r="50"/>
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>4. CHARGE BALANCE VERIFICATION &amp; ERROR TOLERANCE (NCEES CRITERIA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Electro-Neutrality Metric</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Calculated Value</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Standard Criterion / Formula</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Design Status / Exam Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>Total Cation Equivalent Concentration</t>
+        </is>
+      </c>
+      <c r="B53" s="30">
+        <f>B44</f>
+        <v/>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>meq/L</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>Σ Cations from Section 3</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>Total Anion Equivalent Concentration</t>
+        </is>
+      </c>
+      <c r="B54" s="30">
+        <f>B49</f>
+        <v/>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>meq/L</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>Σ Anions from Section 3</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>Net Absolute Charge Difference (|ΣC - ΣA|)</t>
+        </is>
+      </c>
+      <c r="B55" s="30">
+        <f>ABS(B53 - B54)</f>
+        <v/>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>meq/L</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>|Σ Cations - Σ Anions|</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>Normalized Charge Balance Error (% E_cb)</t>
+        </is>
+      </c>
+      <c r="B56" s="30">
+        <f>(B55 / (B53 + B54)) * 100</f>
+        <v/>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>E_cb = |ΣC - ΣA| / (ΣC + ΣA) × 100%</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>Standard Permissible Balance Error Limit</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>Standard acceptable analytical threshold = ±5.0%</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>ELECTRO-NEUTRALITY CODE CHECK</t>
+        </is>
+      </c>
+      <c r="B58" s="57">
+        <f>IF(B56&lt;=B57, "BALANCED (Within ±5%)", IF(B53&gt;B54, "NOT BALANCED (Cations Higher)", "NOT BALANCED (Anions Higher)"))</f>
+        <v/>
+      </c>
+      <c r="C58" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="70" t="inlineStr">
+        <is>
+          <t>NCEES Problem #92 Diagnostic Check</t>
+        </is>
+      </c>
+      <c r="E58" s="71">
+        <f>IF(B56&lt;=B57, "PASS - BALANCED WATER ANALYSIS", "FAIL - ANALYSIS UNBALANCED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59"/>
+    <row r="60" ht="24" customHeight="1">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>5. HARDNESS &amp; STOICHIOMETRIC REAGENTS (AS CaCO3 EQUIVALENTS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Water Chemistry Parameter</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Design Value</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Governing Stoichiometric Equation</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>Total Hardness (TH) as CaCO₃</t>
+        </is>
+      </c>
+      <c r="B62" s="30">
+        <f>(F40 + F41) * 50.0435</f>
+        <v/>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>mg/L as CaCO₃</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>TH = (meq/L Ca²⁺ + meq/L Mg²⁺) × EW(CaCO₃)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>Calcium Hardness (CH) as CaCO₃</t>
+        </is>
+      </c>
+      <c r="B63" s="30">
+        <f>F40 * 50.0435</f>
+        <v/>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>mg/L as CaCO₃</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>CH = meq/L Ca²⁺ × 50.0435 mg/meq</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>Magnesium Hardness (MH) as CaCO₃</t>
+        </is>
+      </c>
+      <c r="B64" s="30">
+        <f>F41 * 50.0435</f>
+        <v/>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>mg/L as CaCO₃</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>MH = meq/L Mg²⁺ × 50.0435 mg/meq</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>Total Alkalinity (Alk) as CaCO₃</t>
+        </is>
+      </c>
+      <c r="B65" s="30">
+        <f>F45 * 50.0435</f>
+        <v/>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>mg/L as CaCO₃</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>Alk = meq/L HCO₃⁻ × 50.0435 mg/meq (pH 4.5-8.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>Carbonate Hardness (CH)</t>
+        </is>
+      </c>
+      <c r="B66" s="30">
+        <f>MIN(B62, B65)</f>
+        <v/>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>mg/L as CaCO₃</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>CH = min(Total Hardness, Total Alkalinity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>Non-Carbonate Hardness (NCH)</t>
+        </is>
+      </c>
+      <c r="B67" s="30">
+        <f>MAX(0, B62 - B65)</f>
+        <v/>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>mg/L as CaCO₃</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>NCH = max(0, Total Hardness - Total Alkalinity)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9438,7 +11125,7 @@
         </is>
       </c>
       <c r="B9" s="33">
-        <f>B4 * B5 * B6</f>
+        <f>B6 * B7 * B8</f>
         <v/>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -9479,7 +11166,7 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>B7 * (B8 * 60)</f>
+        <f>B9 * (B10 * 60)</f>
         <v/>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -9500,7 +11187,7 @@
         </is>
       </c>
       <c r="B12" s="30">
-        <f>B9 / 43560</f>
+        <f>B11 / 43560</f>
         <v/>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -9588,27 +11275,27 @@
         <v>1</v>
       </c>
       <c r="B17" s="22">
-        <f>120 + 2*3*A14</f>
+        <f>120 + 2*3*A17</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>60 + 2*3*A14</f>
+        <f>60 + 2*3*A17</f>
         <v/>
       </c>
       <c r="D17" s="22">
-        <f>B14 * C14</f>
+        <f>B17 * C17</f>
         <v/>
       </c>
       <c r="E17" s="22">
-        <f>(1/3)*(D13 + D14 + SQRT(D13*D14))</f>
+        <f>(1/3)*(D16 + D17 + SQRT(D16*D17))</f>
         <v/>
       </c>
       <c r="F17" s="20">
-        <f>E14</f>
+        <f>E17</f>
         <v/>
       </c>
       <c r="G17" s="20">
-        <f>F14/43560</f>
+        <f>F17/43560</f>
         <v/>
       </c>
     </row>
@@ -9617,27 +11304,27 @@
         <v>2</v>
       </c>
       <c r="B18" s="22">
-        <f>120 + 2*3*A15</f>
+        <f>120 + 2*3*A18</f>
         <v/>
       </c>
       <c r="C18" s="20">
-        <f>60 + 2*3*A15</f>
+        <f>60 + 2*3*A18</f>
         <v/>
       </c>
       <c r="D18" s="22">
-        <f>B15 * C15</f>
+        <f>B18 * C18</f>
         <v/>
       </c>
       <c r="E18" s="22">
-        <f>(1/3)*(D14 + D15 + SQRT(D14*D15))</f>
+        <f>(1/3)*(D17 + D18 + SQRT(D17*D18))</f>
         <v/>
       </c>
       <c r="F18" s="20">
-        <f>F14 + E15</f>
+        <f>F17 + E18</f>
         <v/>
       </c>
       <c r="G18" s="20">
-        <f>F15/43560</f>
+        <f>F18/43560</f>
         <v/>
       </c>
     </row>
@@ -9646,27 +11333,27 @@
         <v>3</v>
       </c>
       <c r="B19" s="22">
-        <f>120 + 2*3*A16</f>
+        <f>120 + 2*3*A19</f>
         <v/>
       </c>
       <c r="C19" s="20">
-        <f>60 + 2*3*A16</f>
+        <f>60 + 2*3*A19</f>
         <v/>
       </c>
       <c r="D19" s="22">
-        <f>B16 * C16</f>
+        <f>B19 * C19</f>
         <v/>
       </c>
       <c r="E19" s="22">
-        <f>(1/3)*(D15 + D16 + SQRT(D15*D16))</f>
+        <f>(1/3)*(D18 + D19 + SQRT(D18*D19))</f>
         <v/>
       </c>
       <c r="F19" s="20">
-        <f>F15 + E16</f>
+        <f>F18 + E19</f>
         <v/>
       </c>
       <c r="G19" s="20">
-        <f>F16/43560</f>
+        <f>F19/43560</f>
         <v/>
       </c>
     </row>
@@ -9675,27 +11362,27 @@
         <v>4</v>
       </c>
       <c r="B20" s="22">
-        <f>120 + 2*3*A17</f>
+        <f>120 + 2*3*A20</f>
         <v/>
       </c>
       <c r="C20" s="20">
-        <f>60 + 2*3*A17</f>
+        <f>60 + 2*3*A20</f>
         <v/>
       </c>
       <c r="D20" s="22">
-        <f>B17 * C17</f>
+        <f>B20 * C20</f>
         <v/>
       </c>
       <c r="E20" s="22">
-        <f>(1/3)*(D16 + D17 + SQRT(D16*D17))</f>
+        <f>(1/3)*(D19 + D20 + SQRT(D19*D20))</f>
         <v/>
       </c>
       <c r="F20" s="20">
-        <f>F16 + E17</f>
+        <f>F19 + E20</f>
         <v/>
       </c>
       <c r="G20" s="20">
-        <f>F17/43560</f>
+        <f>F20/43560</f>
         <v/>
       </c>
     </row>
@@ -9704,27 +11391,27 @@
         <v>5</v>
       </c>
       <c r="B21" s="22">
-        <f>120 + 2*3*A18</f>
+        <f>120 + 2*3*A21</f>
         <v/>
       </c>
       <c r="C21" s="20">
-        <f>60 + 2*3*A18</f>
+        <f>60 + 2*3*A21</f>
         <v/>
       </c>
       <c r="D21" s="22">
-        <f>B18 * C18</f>
+        <f>B21 * C21</f>
         <v/>
       </c>
       <c r="E21" s="22">
-        <f>(1/3)*(D17 + D18 + SQRT(D17*D18))</f>
+        <f>(1/3)*(D20 + D21 + SQRT(D20*D21))</f>
         <v/>
       </c>
       <c r="F21" s="20">
-        <f>F17 + E18</f>
+        <f>F20 + E21</f>
         <v/>
       </c>
       <c r="G21" s="20">
-        <f>F18/43560</f>
+        <f>F21/43560</f>
         <v/>
       </c>
     </row>
@@ -9733,27 +11420,27 @@
         <v>6</v>
       </c>
       <c r="B22" s="22">
-        <f>120 + 2*3*A19</f>
+        <f>120 + 2*3*A22</f>
         <v/>
       </c>
       <c r="C22" s="20">
-        <f>60 + 2*3*A19</f>
+        <f>60 + 2*3*A22</f>
         <v/>
       </c>
       <c r="D22" s="22">
-        <f>B19 * C19</f>
+        <f>B22 * C22</f>
         <v/>
       </c>
       <c r="E22" s="22">
-        <f>(1/3)*(D18 + D19 + SQRT(D18*D19))</f>
+        <f>(1/3)*(D21 + D22 + SQRT(D21*D22))</f>
         <v/>
       </c>
       <c r="F22" s="20">
-        <f>F18 + E19</f>
+        <f>F21 + E22</f>
         <v/>
       </c>
       <c r="G22" s="20">
-        <f>F19/43560</f>
+        <f>F22/43560</f>
         <v/>
       </c>
     </row>
@@ -9874,7 +11561,7 @@
         </is>
       </c>
       <c r="B29" s="19">
-        <f>B21 / (B22 * SQRT(2 * 32.174 * B23))</f>
+        <f>B26 / (B27 * SQRT(2 * 32.174 * B28))</f>
         <v/>
       </c>
       <c r="C29" s="13" t="inlineStr">
@@ -9900,7 +11587,7 @@
         </is>
       </c>
       <c r="B30" s="30">
-        <f>SQRT(4 * B24 / PI()) * 12</f>
+        <f>SQRT(4 * B29 / PI()) * 12</f>
         <v/>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -9926,7 +11613,7 @@
         </is>
       </c>
       <c r="B31" s="31">
-        <f>F19</f>
+        <f>F22</f>
         <v/>
       </c>
       <c r="C31" s="28" t="inlineStr">
@@ -9940,7 +11627,7 @@
         </is>
       </c>
       <c r="E31" s="32">
-        <f>IF(F19&gt;=B9*0.6, "PASS - DETENTION VOLUME ADEQUATE", "FAIL - EXPAND POND")</f>
+        <f>IF(F22&gt;=B11*0.6, "PASS - DETENTION VOLUME ADEQUATE", "FAIL - EXPAND POND")</f>
         <v/>
       </c>
     </row>
@@ -9964,7 +11651,7 @@
         </is>
       </c>
       <c r="E32" s="29">
-        <f>IF(B27&gt;=1.0, "PASS - FREEBOARD COMPLIANT", "FAIL - OVERTOPPING RISK")</f>
+        <f>IF(B32&gt;=1.0, "PASS - FREEBOARD COMPLIANT", "FAIL - OVERTOPPING RISK")</f>
         <v/>
       </c>
     </row>
@@ -10239,7 +11926,7 @@
         </is>
       </c>
       <c r="B17" s="22">
-        <f>(B5 * B7) / B6</f>
+        <f>(B7 * B9) / B8</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -10260,7 +11947,7 @@
         </is>
       </c>
       <c r="B18" s="30">
-        <f>SQRT(4 * B13 * B10)</f>
+        <f>SQRT(4 * B17 * B12)</f>
         <v/>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -10281,7 +11968,7 @@
         </is>
       </c>
       <c r="B19" s="37">
-        <f>B8 / B14</f>
+        <f>B10 / B18</f>
         <v/>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -10302,7 +11989,7 @@
         </is>
       </c>
       <c r="B20" s="37">
-        <f>B9 / B14</f>
+        <f>B11 / B18</f>
         <v/>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -10323,7 +12010,7 @@
         </is>
       </c>
       <c r="B21" s="37">
-        <f>4 * B15 * B16 * (1 - 0.33*(B15^2 + B16^2))</f>
+        <f>4 * B19 * B20 * (1 - 0.33*(B19^2 + B20^2))</f>
         <v/>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -10344,7 +12031,7 @@
         </is>
       </c>
       <c r="B22" s="30">
-        <f>(B4 / (4 * B5 * B7 / B6)) * B14^2 * B17</f>
+        <f>(B6 / (4 * B7 * B9 / B8)) * B18^2 * B21</f>
         <v/>
       </c>
       <c r="C22" s="13" t="inlineStr">
@@ -10365,7 +12052,7 @@
         </is>
       </c>
       <c r="B23" s="30">
-        <f>SQRT(B7^2 + 2*B7*B18) - B7</f>
+        <f>SQRT(B9^2 + 2*B9*B22) - B9</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -10447,7 +12134,7 @@
         </is>
       </c>
       <c r="B28" s="27">
-        <f>B11 - B19</f>
+        <f>B13 - B23</f>
         <v/>
       </c>
       <c r="C28" s="28" t="inlineStr">
@@ -10461,7 +12148,7 @@
         </is>
       </c>
       <c r="E28" s="29">
-        <f>IF((B11-B19)&gt;=2.0, "PASS - SHWT SEPARATION MAINTAINED", "FAIL - GROUNDWATER BREAKOUT RISK")</f>
+        <f>IF((B13-B23)&gt;=2.0, "PASS - SHWT SEPARATION MAINTAINED", "FAIL - GROUNDWATER BREAKOUT RISK")</f>
         <v/>
       </c>
     </row>
@@ -10472,7 +12159,7 @@
         </is>
       </c>
       <c r="B29" s="39">
-        <f>(B11 - B19) * 12</f>
+        <f>(B13 - B23) * 12</f>
         <v/>
       </c>
       <c r="C29" s="28" t="inlineStr">
@@ -10486,7 +12173,7 @@
         </is>
       </c>
       <c r="E29" s="41">
-        <f>IF(((B11-B19)*12)&gt;=24.0, "PASS", "FAIL")</f>
+        <f>IF(((B13-B23)*12)&gt;=24.0, "PASS - SHWT &gt;= 24 INCHES", "FAIL - SHWT VIOLATION")</f>
         <v/>
       </c>
     </row>
@@ -10651,7 +12338,7 @@
         </is>
       </c>
       <c r="B10" s="22">
-        <f>B4^2 / (15 * (B6 + B7))</f>
+        <f>B6^2 / (15 * (B8 + B9))</f>
         <v/>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -10692,7 +12379,7 @@
         </is>
       </c>
       <c r="B12" s="30">
-        <f>5729.578 / B9</f>
+        <f>5729.578 / B11</f>
         <v/>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -10713,7 +12400,7 @@
         </is>
       </c>
       <c r="B13" s="33">
-        <f>B9 * TAN(RADIANS(B5 / 2))</f>
+        <f>B11 * TAN(RADIANS(B7 / 2))</f>
         <v/>
       </c>
       <c r="C13" s="13" t="inlineStr">
@@ -10734,7 +12421,7 @@
         </is>
       </c>
       <c r="B14" s="33">
-        <f>(PI() * B9 * B5) / 180</f>
+        <f>(PI() * B11 * B7) / 180</f>
         <v/>
       </c>
       <c r="C14" s="13" t="inlineStr">
@@ -10755,7 +12442,7 @@
         </is>
       </c>
       <c r="B15" s="30">
-        <f>B9 * (1/COS(RADIANS(B5/2)) - 1)</f>
+        <f>B11 * (1/COS(RADIANS(B7/2)) - 1)</f>
         <v/>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -10776,7 +12463,7 @@
         </is>
       </c>
       <c r="B16" s="30">
-        <f>B9 * (1 - COS(RADIANS(B5/2)))</f>
+        <f>B11 * (1 - COS(RADIANS(B7/2)))</f>
         <v/>
       </c>
       <c r="C16" s="13" t="inlineStr">
@@ -10887,7 +12574,7 @@
         </is>
       </c>
       <c r="B23" s="22">
-        <f>1.47 * B4 * B16</f>
+        <f>1.47 * B6 * B20</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -10908,7 +12595,7 @@
         </is>
       </c>
       <c r="B24" s="22">
-        <f>B4^2 / (30 * (B17/32.174 + B18))</f>
+        <f>B6^2 / (30 * (B21/32.174 + B22))</f>
         <v/>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -10929,7 +12616,7 @@
         </is>
       </c>
       <c r="B25" s="22">
-        <f>B19 + B20</f>
+        <f>B23 + B24</f>
         <v/>
       </c>
       <c r="C25" s="13" t="inlineStr">
@@ -10994,7 +12681,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="30">
-        <f>B24 * C24 * D24</f>
+        <f>B29 * C29 * D29</f>
         <v/>
       </c>
     </row>
@@ -11014,7 +12701,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="30">
-        <f>B25 * C25 * D25</f>
+        <f>B30 * C30 * D30</f>
         <v/>
       </c>
     </row>
@@ -11034,7 +12721,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="30">
-        <f>B26 * C26 * D26</f>
+        <f>B31 * C31 * D31</f>
         <v/>
       </c>
     </row>
@@ -11058,7 +12745,7 @@
         </is>
       </c>
       <c r="E32" s="45">
-        <f>E24 + E25 + E26</f>
+        <f>E29 + E30 + E31</f>
         <v/>
       </c>
     </row>
@@ -11307,7 +12994,7 @@
         </is>
       </c>
       <c r="B15" s="30">
-        <f>ABS(B9 - B10)</f>
+        <f>ABS(B14 - B13)</f>
         <v/>
       </c>
       <c r="C15" s="13" t="inlineStr">
@@ -11348,7 +13035,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>B12 * TAN(RADIANS(B11 / 2))</f>
+        <f>B16 * TAN(RADIANS(B15 / 2))</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -11369,7 +13056,7 @@
         </is>
       </c>
       <c r="B18" s="30">
-        <f>B8 - B13</f>
+        <f>B12 - B17</f>
         <v/>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -11390,7 +13077,7 @@
         </is>
       </c>
       <c r="B19" s="30">
-        <f>(PI() * B12 * B11) / 180</f>
+        <f>(PI() * B16 * B15) / 180</f>
         <v/>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -11441,11 +13128,11 @@
         </is>
       </c>
       <c r="B23" s="33">
-        <f>B8 * B8</f>
+        <f>B12 * B12</f>
         <v/>
       </c>
       <c r="C23" s="20">
-        <f>B18 / 43560</f>
+        <f>B23 / 43560</f>
         <v/>
       </c>
       <c r="D23" s="34" t="inlineStr">
@@ -11461,11 +13148,11 @@
         </is>
       </c>
       <c r="B24" s="30">
-        <f>B12*B13 - 0.5*B12^2*RADIANS(B11)</f>
+        <f>B16*B17 - 0.5*B16^2*RADIANS(B15)</f>
         <v/>
       </c>
       <c r="C24" s="20">
-        <f>B19 / 43560</f>
+        <f>B24 / 43560</f>
         <v/>
       </c>
       <c r="D24" s="14" t="inlineStr">
@@ -11481,11 +13168,11 @@
         </is>
       </c>
       <c r="B25" s="48">
-        <f>B18 - B19</f>
+        <f>B23 - B24</f>
         <v/>
       </c>
       <c r="C25" s="25">
-        <f>B20 / 43560</f>
+        <f>B25 / 43560</f>
         <v/>
       </c>
       <c r="D25" s="49" t="inlineStr">
@@ -11635,7 +13322,7 @@
         </is>
       </c>
       <c r="B9" s="37">
-        <f>(PI()/4) * (B4/12)^2</f>
+        <f>(PI()/4) * (B6/12)^2</f>
         <v/>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -11656,7 +13343,7 @@
         </is>
       </c>
       <c r="B10" s="37">
-        <f>(B4/12) / 4</f>
+        <f>(B6/12) / 4</f>
         <v/>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -11677,7 +13364,7 @@
         </is>
       </c>
       <c r="B11" s="30">
-        <f>(1.486 / B5) * B8^(2/3) * SQRT(B6)</f>
+        <f>(1.486 / B7) * B10^(2/3) * SQRT(B8)</f>
         <v/>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -11698,7 +13385,7 @@
         </is>
       </c>
       <c r="B12" s="22">
-        <f>B9 * B7 * 448.83</f>
+        <f>B11 * B9 * 448.83</f>
         <v/>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -11719,7 +13406,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>B9</f>
+        <f>B11</f>
         <v/>
       </c>
       <c r="C13" s="28" t="inlineStr">
@@ -11733,7 +13420,7 @@
         </is>
       </c>
       <c r="E13" s="29">
-        <f>IF(B9&gt;=2.0, "PASS - SCOURING VELOCITY MAINTAINED", "FAIL - SLUGGING RISK")</f>
+        <f>IF(B11&gt;=2.0, "PASS - SCOURING VELOCITY MAINTAINED", "FAIL - SLUGGING RISK")</f>
         <v/>
       </c>
     </row>
@@ -11834,7 +13521,7 @@
         </is>
       </c>
       <c r="B20" s="22">
-        <f>(B15 * B14) / 4</f>
+        <f>(B19 * B18) / 4</f>
         <v/>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -11855,7 +13542,7 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>B16 / 7.48052</f>
+        <f>B20 / 7.48052</f>
         <v/>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -11896,7 +13583,7 @@
         </is>
       </c>
       <c r="B23" s="30">
-        <f>(PI()/4) * B18^2</f>
+        <f>(PI()/4) * B22^2</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -11917,7 +13604,7 @@
         </is>
       </c>
       <c r="B24" s="30">
-        <f>B17 / B19</f>
+        <f>B21 / B23</f>
         <v/>
       </c>
       <c r="C24" s="13" t="inlineStr">
@@ -12048,7 +13735,7 @@
         </is>
       </c>
       <c r="B32" s="30">
-        <f>(B14 / 448.83) / ((PI()/4)*(B22/12)^2)</f>
+        <f>(B18 / 448.83) / ((PI()/4)*(B28/12)^2)</f>
         <v/>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -12069,7 +13756,7 @@
         </is>
       </c>
       <c r="B33" s="30">
-        <f>10.44 * B23 * B14^1.852 / (B24^1.852 * B22^4.87)</f>
+        <f>10.44 * B29 * B18^1.852 / (B30^1.852 * B28^4.87)</f>
         <v/>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -12090,7 +13777,7 @@
         </is>
       </c>
       <c r="B34" s="30">
-        <f>0.10 * B27</f>
+        <f>0.10 * B33</f>
         <v/>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -12111,7 +13798,7 @@
         </is>
       </c>
       <c r="B35" s="30">
-        <f>B25 + B27 + B28</f>
+        <f>B31 + B33 + B34</f>
         <v/>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -12152,7 +13839,7 @@
         </is>
       </c>
       <c r="B37" s="30">
-        <f>(B14 * B29) / (3960 * B30)</f>
+        <f>(B18 * B35) / (3960 * B36)</f>
         <v/>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -12173,7 +13860,7 @@
         </is>
       </c>
       <c r="B38" s="52">
-        <f>ROUNDUP(B31 * 1.15, 0)</f>
+        <f>ROUNDUP(B37 * 1.15, 0)</f>
         <v/>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -12328,7 +14015,7 @@
         </is>
       </c>
       <c r="B9" s="30">
-        <f>135 / (B6 + 18)^0.82</f>
+        <f>135 / (B8 + 18)^0.82</f>
         <v/>
       </c>
       <c r="C9" s="13" t="inlineStr">
@@ -12349,7 +14036,7 @@
         </is>
       </c>
       <c r="B10" s="33">
-        <f>B4 * B5 * B7</f>
+        <f>B6 * B7 * B9</f>
         <v/>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -12460,7 +14147,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>( (B8 * B13) / (0.56 * B12^(5/3) * B11^0.5) )^(3/8)</f>
+        <f>((B10 * B16) / (0.56 * B15^(5/3) * B14^0.5))^(3/8)</f>
         <v/>
       </c>
       <c r="C17" s="13" t="inlineStr">
@@ -12494,7 +14181,7 @@
         </is>
       </c>
       <c r="E18" s="29">
-        <f>IF(B14&lt;=B15, "PASS - GUTTER SPREAD WITHIN SHOULDER", "FAIL - TRAFFIC LANE INUNDATED")</f>
+        <f>IF(B17&lt;=B18, "PASS - GUTTER SPREAD WITHIN SHOULDER", "FAIL - TRAFFIC LANE INUNDATED")</f>
         <v/>
       </c>
     </row>
@@ -12615,7 +14302,7 @@
         </is>
       </c>
       <c r="B26" s="30">
-        <f>(B18/12) * ( 1.0 + 0.038 * (B8 / ((PI()/4)*(B18/12)^2 * SQRT(B18/12)))^1.5 )</f>
+        <f>(B22/12) * (1.0 + 0.038 * (B10 / ((PI()/4)*(B22/12)^2 * SQRT(B22/12)))^1.5)</f>
         <v/>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -12636,7 +14323,7 @@
         </is>
       </c>
       <c r="B27" s="30">
-        <f>2.5 + (1 + 0.5 + 29*B21^2*B19/((B18/12)^(4/3))) * ((B8/((PI()/4)*(B18/12)^2))^2 / (2*32.174)) - B19*B20</f>
+        <f>2.5 + (1 + 0.5 + 29*B25^2*B23/((B22/12)^(4/3))) * ((B10/((PI()/4)*(B22/12)^2))^2 / (2*32.174)) - B24*B23</f>
         <v/>
       </c>
       <c r="C27" s="13" t="inlineStr">
@@ -12657,7 +14344,7 @@
         </is>
       </c>
       <c r="B28" s="30">
-        <f>MAX(B22, B23)</f>
+        <f>MAX(B26, B27)</f>
         <v/>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -12718,7 +14405,7 @@
         </is>
       </c>
       <c r="B31" s="27">
-        <f>B25 - (B26 + B24)</f>
+        <f>B29 - (B30 + B28)</f>
         <v/>
       </c>
       <c r="C31" s="28" t="inlineStr">
@@ -12732,7 +14419,7 @@
         </is>
       </c>
       <c r="E31" s="29">
-        <f>IF((B25-(B26+B24))&gt;=1.0, "PASS - FREEBOARD &gt;= 1.0 FT", "FAIL - ROADWAY OVERTOPPING RISK")</f>
+        <f>IF((B29-(B30+B28))&gt;=1.0, "PASS - FREEBOARD &gt;= 1.0 FT", "FAIL - ROADWAY OVERTOPPING RISK")</f>
         <v/>
       </c>
     </row>
@@ -13027,7 +14714,7 @@
         </is>
       </c>
       <c r="B18" s="30">
-        <f>4 * B4</f>
+        <f>4 * B6</f>
         <v/>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -13048,7 +14735,7 @@
         </is>
       </c>
       <c r="B19" s="30">
-        <f>B4 * B4</f>
+        <f>B6 * B6</f>
         <v/>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -13069,7 +14756,7 @@
         </is>
       </c>
       <c r="B20" s="22">
-        <f>B8 * B7 * B13 * B6</f>
+        <f>B10 * B9 * B18 * B8</f>
         <v/>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -13090,7 +14777,7 @@
         </is>
       </c>
       <c r="B21" s="22">
-        <f>(1 - SIN(RADIANS(B10))) * TAN(RADIANS(0.75*B10)) * B11 * B13 * B9</f>
+        <f>(1 - SIN(RADIANS(B12))) * TAN(RADIANS(0.75*B12)) * B13 * B18 * B11</f>
         <v/>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -13111,7 +14798,7 @@
         </is>
       </c>
       <c r="B22" s="30">
-        <f>(B15 + B16) / 1000</f>
+        <f>(B20 + B21) / 1000</f>
         <v/>
       </c>
       <c r="C22" s="13" t="inlineStr">
@@ -13132,7 +14819,7 @@
         </is>
       </c>
       <c r="B23" s="30">
-        <f>(B11 * B12 * B14) / 1000</f>
+        <f>(B13 * B14 * B19) / 1000</f>
         <v/>
       </c>
       <c r="C23" s="13" t="inlineStr">
@@ -13153,7 +14840,7 @@
         </is>
       </c>
       <c r="B24" s="45">
-        <f>B17 + B18</f>
+        <f>B22 + B23</f>
         <v/>
       </c>
       <c r="C24" s="54" t="inlineStr">
@@ -13174,7 +14861,7 @@
         </is>
       </c>
       <c r="B25" s="30">
-        <f>B19 / 2.5</f>
+        <f>B24 / 2.5</f>
         <v/>
       </c>
       <c r="C25" s="13" t="inlineStr">
@@ -13195,7 +14882,7 @@
         </is>
       </c>
       <c r="B26" s="30">
-        <f>B20 / 2.0</f>
+        <f>B25 / 2.0</f>
         <v/>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -13306,7 +14993,7 @@
         </is>
       </c>
       <c r="B33" s="37">
-        <f>1 - (DEGREES(ATAN(B4 / B26)) / 90) * (((B24-1)*B25 + (B25-1)*B24) / (B24 * B25))</f>
+        <f>1 - (DEGREES(ATAN(B6 / B32)) / 90) * (((B31-1)*B30 + (B30-1)*B31) / (B30 * B31))</f>
         <v/>
       </c>
       <c r="C33" s="13" t="inlineStr">
@@ -13327,7 +15014,7 @@
         </is>
       </c>
       <c r="B34" s="22">
-        <f>B24 * B25 * B20 * B27</f>
+        <f>B30 * B31 * B25 * B33</f>
         <v/>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -13348,7 +15035,7 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>B28 / 2.0</f>
+        <f>B34 / 2.0</f>
         <v/>
       </c>
       <c r="C35" s="54" t="inlineStr">

</xml_diff>